<commit_message>
add automatic ATM emails
</commit_message>
<xml_diff>
--- a/Excel Files/COMP_STATEMENT.xlsx
+++ b/Excel Files/COMP_STATEMENT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28575" yWindow="1020" windowWidth="24705" windowHeight="18810" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="51480" yWindow="3555" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="STATEMENT" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,13 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +78,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -112,7 +117,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -399,6 +404,64 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -421,7 +484,7 @@
     <border>
       <left/>
       <right/>
-      <top style="hair">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -429,30 +492,30 @@
     </border>
     <border>
       <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="hair">
         <color indexed="64"/>
       </right>
       <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -499,7 +562,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -509,12 +572,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,12 +590,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -547,11 +598,33 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,31 +643,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -693,7 +767,7 @@
       <col>6</col>
       <colOff>873348</colOff>
       <row>3</row>
-      <rowOff>33793</rowOff>
+      <rowOff>180998</rowOff>
     </to>
     <pic>
       <nvPicPr>
@@ -993,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K45"/>
+  <dimension ref="A2:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="0.7109375" customWidth="1" style="1" min="1" max="1"/>
@@ -1006,6 +1080,7 @@
     <col width="10.28515625" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1" ht="3.95" customHeight="1"/>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -1013,6 +1088,7 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="3.95" customHeight="1"/>
     <row r="4">
       <c r="B4" s="2">
         <f>info!B1</f>
@@ -1031,114 +1107,119 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" thickBot="1"/>
+    <row r="7" ht="3.95" customHeight="1"/>
+    <row r="8" ht="3.95" customHeight="1" thickBot="1"/>
     <row r="9">
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>Sales Performance</t>
         </is>
       </c>
-      <c r="C9" s="30" t="n"/>
+      <c r="C9" s="34" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="E9" s="32" t="inlineStr">
         <is>
           <t>Final Payment</t>
         </is>
       </c>
-      <c r="F9" s="29" t="n"/>
-      <c r="G9" s="30" t="n"/>
+      <c r="F9" s="33" t="n"/>
+      <c r="G9" s="34" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="35" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Level 1 Sales</t>
         </is>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="19">
         <f>_xlfn.XLOOKUP("L1_REV", payout!$G:$G, payout!$F:$F)</f>
         <v/>
       </c>
-      <c r="E10" s="35" t="inlineStr">
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>Level 1 Payout</t>
         </is>
       </c>
-      <c r="F10" s="27" t="n"/>
+      <c r="F10" s="31" t="n"/>
       <c r="G10" s="6">
         <f>_xlfn.XLOOKUP("L1_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
-      <c r="K10" s="19">
+      <c r="K10" s="15">
         <f>C10*0.15</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" thickBot="1">
       <c r="A11" s="5" t="n"/>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>Level 2 Sales</t>
         </is>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="21">
         <f>_xlfn.XLOOKUP("L2_REV", payout!$G:$G, payout!$F:$F)</f>
         <v/>
       </c>
-      <c r="E11" s="35" t="inlineStr">
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="38" t="inlineStr">
         <is>
           <t>Level 2 Payout</t>
         </is>
       </c>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="14">
+      <c r="F11" s="31" t="n"/>
+      <c r="G11" s="12">
         <f>(_xlfn.XLOOKUP("L2_PO",payout!G:G,payout!F:F))</f>
         <v/>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="15">
         <f>C11*0.2</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Total Sales</t>
         </is>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="20">
         <f>SUM(C10:C11)</f>
         <v/>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="F12" s="25" t="n"/>
-      <c r="G12" s="17">
+      <c r="F12" s="29" t="n"/>
+      <c r="G12" s="13">
         <f>SUM(G10:G11)</f>
         <v/>
       </c>
-      <c r="K12" s="19" t="n"/>
+      <c r="K12" s="15" t="n"/>
     </row>
     <row r="13" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>Q1 Threshold</t>
-        </is>
-      </c>
-      <c r="C13" s="41">
-        <f>info!B7</f>
-        <v/>
-      </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>Other Adjustments</t>
-        </is>
-      </c>
-      <c r="F13" s="37" t="n"/>
-      <c r="G13" s="13">
-        <f>_xlfn.IFNA(_xlfn.XLOOKUP("ADJUSTMENTS", payout!G:G,payout!F:F), 0)</f>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>QTD Sales</t>
+        </is>
+      </c>
+      <c r="C13" s="18">
+        <f>_xlfn.IFNA(_xlfn.XLOOKUP("QTD_SALES", payout!G:G,payout!F:F), 0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Adjustments</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="11">
+        <f>_xlfn.IFNA(_xlfn.XLOOKUP("ADJUSTMENTS", payout!G:G,payout!F:F), 0) + _xlfn.IFNA(_xlfn.XLOOKUP("T-SPLIT", payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
@@ -1147,651 +1228,672 @@
         <f>IF(G14&lt;0, 1, 0)</f>
         <v/>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>CS Deduction</t>
         </is>
       </c>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="13">
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="11">
         <f>IFERROR(-_xlfn.XLOOKUP("CS_DEDUCTION", payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" thickBot="1">
+    <row r="15" ht="16.5" customHeight="1">
       <c r="D15" s="5">
-        <f>IF(G15&gt;0, IF(G15&gt;G12, 1, 0), 0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="40" t="inlineStr">
+        <f>IF(G15&gt;0, 1, 0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="43" t="inlineStr">
+        <is>
+          <t>Program Accel</t>
+        </is>
+      </c>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="11">
+        <f>IFERROR(_xlfn.XLOOKUP("PROGRAM_ACCEL_PO",payout!G:G,payout!F:F), 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="16.5" customHeight="1">
+      <c r="D16" s="5">
+        <f>IF(G16&gt;0, 1, 0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>Implant Ratio Accel</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="11">
+        <f>IFERROR(_xlfn.XLOOKUP("IMPLANT_ACCEL_TRUE_UP",payout!G:G,payout!F:F), 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" thickBot="1">
+      <c r="D17" s="5">
+        <f>IF(G17&gt;0, IF(G17&gt;IFERROR(_xlfn.XLOOKUP("TTL_PO", payout!G:G,payout!F:F), 0), 1, 0), 0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="36" t="inlineStr">
         <is>
           <t>Guarantee Adjustment</t>
         </is>
       </c>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="7">
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP("GUR_AMT",payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="E16" s="24" t="inlineStr">
+    <row r="18" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>Final Payout</t>
         </is>
       </c>
-      <c r="F16" s="25" t="n"/>
-      <c r="G16" s="8">
+      <c r="F18" s="29" t="n"/>
+      <c r="G18" s="26">
         <f>_xlfn.XLOOKUP("PO_AMT", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="E17" s="32" t="inlineStr">
+    <row r="19" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Q3 Threshold</t>
+        </is>
+      </c>
+      <c r="C19" s="23">
+        <f>info!B7</f>
+        <v/>
+      </c>
+      <c r="E19" s="39" t="inlineStr">
         <is>
           <t>YTD Payout</t>
         </is>
       </c>
-      <c r="F17" s="33" t="n"/>
-      <c r="G17" s="22">
+      <c r="F19" s="40" t="n"/>
+      <c r="G19" s="17">
         <f>_xlfn.XLOOKUP("YTD_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="38" t="inlineStr">
+    <row r="20" ht="3.95" customHeight="1"/>
+    <row r="21" ht="3.95" customHeight="1"/>
+    <row r="22">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">Opportunity Detail </t>
         </is>
       </c>
-      <c r="C20" s="39" t="n"/>
-      <c r="D20" s="39" t="n"/>
-      <c r="E20" s="39" t="n"/>
-      <c r="F20" s="39" t="n"/>
-      <c r="G20" s="27" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="34" t="inlineStr">
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="45" t="n"/>
+      <c r="E22" s="45" t="n"/>
+      <c r="F22" s="45" t="n"/>
+      <c r="G22" s="31" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="46" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C21" s="34" t="inlineStr">
-        <is>
-          <t>Payout Type</t>
-        </is>
-      </c>
-      <c r="D21" s="34" t="inlineStr">
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="inlineStr">
         <is>
           <t>Opp Name</t>
         </is>
       </c>
-      <c r="E21" s="27" t="n"/>
-      <c r="F21" s="34" t="inlineStr">
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="46" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="G21" s="34" t="inlineStr">
+      <c r="G23" s="46" t="inlineStr">
         <is>
           <t>Rev Units</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="18">
-        <f>IF(LEN(detail!K2)&lt;1,"",detail!K2)</f>
-        <v/>
-      </c>
-      <c r="C22" s="18">
-        <f>IF(LEN(detail!S2)&lt;1,"", detail!S2)</f>
-        <v/>
-      </c>
-      <c r="D22" s="26">
-        <f>IF(LEN(detail!M2)&lt;1,"",detail!M2)</f>
-        <v/>
-      </c>
-      <c r="E22" s="27" t="n"/>
-      <c r="F22" s="11">
-        <f>DOLLAR(IF(LEN(detail!X2)&lt;1,"",detail!X2), 0) &amp; IF(detail!Y2 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G22" s="26">
-        <f>IF(LEN(detail!W2)&lt;1,"",detail!W2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="18">
-        <f>IF(LEN(detail!K3)&lt;1,"",detail!K3)</f>
-        <v/>
-      </c>
-      <c r="C23" s="18">
-        <f>IF(LEN(detail!S3)&lt;1,"", detail!S3)</f>
-        <v/>
-      </c>
-      <c r="D23" s="26">
-        <f>IF(LEN(detail!M3)&lt;1,"",detail!M3)</f>
-        <v/>
-      </c>
-      <c r="E23" s="27" t="n"/>
-      <c r="F23" s="11">
-        <f>DOLLAR(IF(LEN(detail!X3)&lt;1,"",detail!X3), 0) &amp; IF(detail!Y3 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G23" s="26">
-        <f>IF(LEN(detail!W3)&lt;1,"",detail!W3)</f>
-        <v/>
-      </c>
-    </row>
     <row r="24">
-      <c r="B24" s="18">
-        <f>IF(LEN(detail!K4)&lt;1,"",detail!K4)</f>
-        <v/>
-      </c>
-      <c r="C24" s="18">
-        <f>IF(LEN(detail!S4)&lt;1,"", detail!S4)</f>
-        <v/>
-      </c>
-      <c r="D24" s="26">
-        <f>IF(LEN(detail!M4)&lt;1,"",detail!M4)</f>
-        <v/>
-      </c>
-      <c r="E24" s="27" t="n"/>
-      <c r="F24" s="11">
-        <f>DOLLAR(IF(LEN(detail!X4)&lt;1,"",detail!X4), 0) &amp; IF(detail!Y4 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G24" s="26">
-        <f>IF(LEN(detail!W4)&lt;1,"",detail!W4)</f>
+      <c r="B24" s="14">
+        <f>IF(LEN(detail!O2)&lt;1,"",detail!O2)</f>
+        <v/>
+      </c>
+      <c r="C24" s="14">
+        <f>IF(LEN(detail!W2)&lt;1,"", detail!W2)</f>
+        <v/>
+      </c>
+      <c r="D24" s="30">
+        <f>IF(LEN(detail!Q2)&lt;1,"",detail!Q2)</f>
+        <v/>
+      </c>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE2)&lt;1,"",detail!AE2), 0) &amp; IF(detail!AF2 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G24" s="30">
+        <f>IF(LEN(detail!AA2)&lt;1,"",detail!AB2)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="18">
-        <f>IF(LEN(detail!K5)&lt;1,"",detail!K5)</f>
-        <v/>
-      </c>
-      <c r="C25" s="18">
-        <f>IF(LEN(detail!S5)&lt;1,"", detail!S5)</f>
-        <v/>
-      </c>
-      <c r="D25" s="26">
-        <f>IF(LEN(detail!M5)&lt;1,"",detail!M5)</f>
-        <v/>
-      </c>
-      <c r="E25" s="27" t="n"/>
-      <c r="F25" s="11">
-        <f>DOLLAR(IF(LEN(detail!X5)&lt;1,"",detail!X5), 0) &amp; IF(detail!Y5 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G25" s="26">
-        <f>IF(LEN(detail!W5)&lt;1,"",detail!W5)</f>
+      <c r="B25" s="14">
+        <f>IF(LEN(detail!O3)&lt;1,"",detail!O3)</f>
+        <v/>
+      </c>
+      <c r="C25" s="14">
+        <f>IF(LEN(detail!W3)&lt;1,"", detail!W3)</f>
+        <v/>
+      </c>
+      <c r="D25" s="30">
+        <f>IF(LEN(detail!Q3)&lt;1,"",detail!Q3)</f>
+        <v/>
+      </c>
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE3)&lt;1,"",detail!AE3), 0) &amp; IF(detail!AF3 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G25" s="30">
+        <f>IF(LEN(detail!AA3)&lt;1,"",detail!AB3)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="18">
-        <f>IF(LEN(detail!K6)&lt;1,"",detail!K6)</f>
-        <v/>
-      </c>
-      <c r="C26" s="18">
-        <f>IF(LEN(detail!S6)&lt;1,"", detail!S6)</f>
-        <v/>
-      </c>
-      <c r="D26" s="26">
-        <f>IF(LEN(detail!M6)&lt;1,"",detail!M6)</f>
-        <v/>
-      </c>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="11">
-        <f>DOLLAR(IF(LEN(detail!X6)&lt;1,"",detail!X6), 0) &amp; IF(detail!Y6 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G26" s="26">
-        <f>IF(LEN(detail!W6)&lt;1,"",detail!W6)</f>
+      <c r="B26" s="14">
+        <f>IF(LEN(detail!O4)&lt;1,"",detail!O4)</f>
+        <v/>
+      </c>
+      <c r="C26" s="14">
+        <f>IF(LEN(detail!W4)&lt;1,"", detail!W4)</f>
+        <v/>
+      </c>
+      <c r="D26" s="30">
+        <f>IF(LEN(detail!Q4)&lt;1,"",detail!Q4)</f>
+        <v/>
+      </c>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE4)&lt;1,"",detail!AE4), 0) &amp; IF(detail!AF4 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G26" s="30">
+        <f>IF(LEN(detail!AA4)&lt;1,"",detail!AB4)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="18">
-        <f>IF(LEN(detail!K7)&lt;1,"",detail!K7)</f>
-        <v/>
-      </c>
-      <c r="C27" s="18">
-        <f>IF(LEN(detail!S7)&lt;1,"", detail!S7)</f>
-        <v/>
-      </c>
-      <c r="D27" s="26">
-        <f>IF(LEN(detail!M7)&lt;1,"",detail!M7)</f>
-        <v/>
-      </c>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="11">
-        <f>DOLLAR(IF(LEN(detail!X7)&lt;1,"",detail!X7), 0) &amp; IF(detail!Y7 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G27" s="26">
-        <f>IF(LEN(detail!W7)&lt;1,"",detail!W7)</f>
+      <c r="B27" s="14">
+        <f>IF(LEN(detail!O5)&lt;1,"",detail!O5)</f>
+        <v/>
+      </c>
+      <c r="C27" s="14">
+        <f>IF(LEN(detail!W5)&lt;1,"", detail!W5)</f>
+        <v/>
+      </c>
+      <c r="D27" s="30">
+        <f>IF(LEN(detail!Q5)&lt;1,"",detail!Q5)</f>
+        <v/>
+      </c>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE5)&lt;1,"",detail!AE5), 0) &amp; IF(detail!AF5 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G27" s="30">
+        <f>IF(LEN(detail!AA5)&lt;1,"",detail!AB5)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="18">
-        <f>IF(LEN(detail!K8)&lt;1,"",detail!K8)</f>
-        <v/>
-      </c>
-      <c r="C28" s="18">
-        <f>IF(LEN(detail!S8)&lt;1,"", detail!S8)</f>
-        <v/>
-      </c>
-      <c r="D28" s="26">
-        <f>IF(LEN(detail!M8)&lt;1,"",detail!M8)</f>
-        <v/>
-      </c>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="11">
-        <f>DOLLAR(IF(LEN(detail!X8)&lt;1,"",detail!X8), 0) &amp; IF(detail!Y8 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G28" s="26">
-        <f>IF(LEN(detail!W8)&lt;1,"",detail!W8)</f>
+      <c r="B28" s="14">
+        <f>IF(LEN(detail!O6)&lt;1,"",detail!O6)</f>
+        <v/>
+      </c>
+      <c r="C28" s="14">
+        <f>IF(LEN(detail!W6)&lt;1,"", detail!W6)</f>
+        <v/>
+      </c>
+      <c r="D28" s="30">
+        <f>IF(LEN(detail!Q6)&lt;1,"",detail!Q6)</f>
+        <v/>
+      </c>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE6)&lt;1,"",detail!AE6), 0) &amp; IF(detail!AF6 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G28" s="30">
+        <f>IF(LEN(detail!AA6)&lt;1,"",detail!AB6)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="18">
-        <f>IF(LEN(detail!K9)&lt;1,"",detail!K9)</f>
-        <v/>
-      </c>
-      <c r="C29" s="18">
-        <f>IF(LEN(detail!S9)&lt;1,"", detail!S9)</f>
-        <v/>
-      </c>
-      <c r="D29" s="26">
-        <f>IF(LEN(detail!M9)&lt;1,"",detail!M9)</f>
-        <v/>
-      </c>
-      <c r="E29" s="27" t="n"/>
-      <c r="F29" s="11">
-        <f>DOLLAR(IF(LEN(detail!X9)&lt;1,"",detail!X9), 0) &amp; IF(detail!Y9 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G29" s="26">
-        <f>IF(LEN(detail!W9)&lt;1,"",detail!W9)</f>
+      <c r="B29" s="14">
+        <f>IF(LEN(detail!O7)&lt;1,"",detail!O7)</f>
+        <v/>
+      </c>
+      <c r="C29" s="14">
+        <f>IF(LEN(detail!W7)&lt;1,"", detail!W7)</f>
+        <v/>
+      </c>
+      <c r="D29" s="30">
+        <f>IF(LEN(detail!Q7)&lt;1,"",detail!Q7)</f>
+        <v/>
+      </c>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE7)&lt;1,"",detail!AE7), 0) &amp; IF(detail!AF7 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G29" s="30">
+        <f>IF(LEN(detail!AA7)&lt;1,"",detail!AB7)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="18">
-        <f>IF(LEN(detail!K10)&lt;1,"",detail!K10)</f>
-        <v/>
-      </c>
-      <c r="C30" s="18">
-        <f>IF(LEN(detail!S10)&lt;1,"", detail!S10)</f>
-        <v/>
-      </c>
-      <c r="D30" s="26">
-        <f>IF(LEN(detail!M10)&lt;1,"",detail!M10)</f>
-        <v/>
-      </c>
-      <c r="E30" s="27" t="n"/>
-      <c r="F30" s="11">
-        <f>DOLLAR(IF(LEN(detail!X10)&lt;1,"",detail!X10), 0) &amp; IF(detail!Y10 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G30" s="26">
-        <f>IF(LEN(detail!W10)&lt;1,"",detail!W10)</f>
+      <c r="B30" s="14">
+        <f>IF(LEN(detail!O8)&lt;1,"",detail!O8)</f>
+        <v/>
+      </c>
+      <c r="C30" s="14">
+        <f>IF(LEN(detail!W8)&lt;1,"", detail!W8)</f>
+        <v/>
+      </c>
+      <c r="D30" s="30">
+        <f>IF(LEN(detail!Q8)&lt;1,"",detail!Q8)</f>
+        <v/>
+      </c>
+      <c r="E30" s="31" t="n"/>
+      <c r="F30" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE8)&lt;1,"",detail!AE8), 0) &amp; IF(detail!AF8 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G30" s="30">
+        <f>IF(LEN(detail!AA8)&lt;1,"",detail!AB8)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="18">
-        <f>IF(LEN(detail!K11)&lt;1,"",detail!K11)</f>
-        <v/>
-      </c>
-      <c r="C31" s="18">
-        <f>IF(LEN(detail!S11)&lt;1,"", detail!S11)</f>
-        <v/>
-      </c>
-      <c r="D31" s="26">
-        <f>IF(LEN(detail!M11)&lt;1,"",detail!M11)</f>
-        <v/>
-      </c>
-      <c r="E31" s="27" t="n"/>
-      <c r="F31" s="11">
-        <f>DOLLAR(IF(LEN(detail!X11)&lt;1,"",detail!X11), 0) &amp; IF(detail!Y11 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G31" s="26">
-        <f>IF(LEN(detail!W11)&lt;1,"",detail!W11)</f>
+      <c r="B31" s="14">
+        <f>IF(LEN(detail!O9)&lt;1,"",detail!O9)</f>
+        <v/>
+      </c>
+      <c r="C31" s="14">
+        <f>IF(LEN(detail!W9)&lt;1,"", detail!W9)</f>
+        <v/>
+      </c>
+      <c r="D31" s="30">
+        <f>IF(LEN(detail!Q9)&lt;1,"",detail!Q9)</f>
+        <v/>
+      </c>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE9)&lt;1,"",detail!AE9), 0) &amp; IF(detail!AF9 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G31" s="30">
+        <f>IF(LEN(detail!AA9)&lt;1,"",detail!AB9)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="18">
-        <f>IF(LEN(detail!K12)&lt;1,"",detail!K12)</f>
-        <v/>
-      </c>
-      <c r="C32" s="18">
-        <f>IF(LEN(detail!S12)&lt;1,"", detail!S12)</f>
-        <v/>
-      </c>
-      <c r="D32" s="26">
-        <f>IF(LEN(detail!M12)&lt;1,"",detail!M12)</f>
-        <v/>
-      </c>
-      <c r="E32" s="27" t="n"/>
-      <c r="F32" s="11">
-        <f>DOLLAR(IF(LEN(detail!X12)&lt;1,"",detail!X12), 0) &amp; IF(detail!Y12 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G32" s="26">
-        <f>IF(LEN(detail!W12)&lt;1,"",detail!W12)</f>
+      <c r="B32" s="14">
+        <f>IF(LEN(detail!O10)&lt;1,"",detail!O10)</f>
+        <v/>
+      </c>
+      <c r="C32" s="14">
+        <f>IF(LEN(detail!W10)&lt;1,"", detail!W10)</f>
+        <v/>
+      </c>
+      <c r="D32" s="30">
+        <f>IF(LEN(detail!Q10)&lt;1,"",detail!Q10)</f>
+        <v/>
+      </c>
+      <c r="E32" s="31" t="n"/>
+      <c r="F32" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE10)&lt;1,"",detail!AE10), 0) &amp; IF(detail!AF10 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G32" s="30">
+        <f>IF(LEN(detail!AA10)&lt;1,"",detail!AB10)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="18">
-        <f>IF(LEN(detail!K13)&lt;1,"",detail!K13)</f>
-        <v/>
-      </c>
-      <c r="C33" s="18">
-        <f>IF(LEN(detail!S13)&lt;1,"", detail!S13)</f>
-        <v/>
-      </c>
-      <c r="D33" s="26">
-        <f>IF(LEN(detail!M13)&lt;1,"",detail!M13)</f>
-        <v/>
-      </c>
-      <c r="E33" s="27" t="n"/>
-      <c r="F33" s="11">
-        <f>DOLLAR(IF(LEN(detail!X13)&lt;1,"",detail!X13), 0) &amp; IF(detail!Y13 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G33" s="26">
-        <f>IF(LEN(detail!W13)&lt;1,"",detail!W13)</f>
+      <c r="B33" s="14">
+        <f>IF(LEN(detail!O11)&lt;1,"",detail!O11)</f>
+        <v/>
+      </c>
+      <c r="C33" s="14">
+        <f>IF(LEN(detail!W11)&lt;1,"", detail!W11)</f>
+        <v/>
+      </c>
+      <c r="D33" s="30">
+        <f>IF(LEN(detail!Q11)&lt;1,"",detail!Q11)</f>
+        <v/>
+      </c>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE11)&lt;1,"",detail!AE11), 0) &amp; IF(detail!AF11 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G33" s="30">
+        <f>IF(LEN(detail!AA11)&lt;1,"",detail!AB11)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="18">
-        <f>IF(LEN(detail!K14)&lt;1,"",detail!K14)</f>
-        <v/>
-      </c>
-      <c r="C34" s="18">
-        <f>IF(LEN(detail!S14)&lt;1,"", detail!S14)</f>
-        <v/>
-      </c>
-      <c r="D34" s="26">
-        <f>IF(LEN(detail!M14)&lt;1,"",detail!M14)</f>
-        <v/>
-      </c>
-      <c r="E34" s="27" t="n"/>
-      <c r="F34" s="11">
-        <f>DOLLAR(IF(LEN(detail!X14)&lt;1,"",detail!X14), 0) &amp; IF(detail!Y14 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G34" s="26">
-        <f>IF(LEN(detail!W14)&lt;1,"",detail!W14)</f>
+      <c r="B34" s="14">
+        <f>IF(LEN(detail!O12)&lt;1,"",detail!O12)</f>
+        <v/>
+      </c>
+      <c r="C34" s="14">
+        <f>IF(LEN(detail!W12)&lt;1,"", detail!W12)</f>
+        <v/>
+      </c>
+      <c r="D34" s="30">
+        <f>IF(LEN(detail!Q12)&lt;1,"",detail!Q12)</f>
+        <v/>
+      </c>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE12)&lt;1,"",detail!AE12), 0) &amp; IF(detail!AF12 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G34" s="30">
+        <f>IF(LEN(detail!AA12)&lt;1,"",detail!AB12)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="18">
-        <f>IF(LEN(detail!K15)&lt;1,"",detail!K15)</f>
-        <v/>
-      </c>
-      <c r="C35" s="18">
-        <f>IF(LEN(detail!S15)&lt;1,"", detail!S15)</f>
-        <v/>
-      </c>
-      <c r="D35" s="26">
-        <f>IF(LEN(detail!M15)&lt;1,"",detail!M15)</f>
-        <v/>
-      </c>
-      <c r="E35" s="27" t="n"/>
-      <c r="F35" s="11">
-        <f>DOLLAR(IF(LEN(detail!X15)&lt;1,"",detail!X15), 0) &amp; IF(detail!Y15 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G35" s="26">
-        <f>IF(LEN(detail!W15)&lt;1,"",detail!W15)</f>
+      <c r="B35" s="14">
+        <f>IF(LEN(detail!O13)&lt;1,"",detail!O13)</f>
+        <v/>
+      </c>
+      <c r="C35" s="14">
+        <f>IF(LEN(detail!W13)&lt;1,"", detail!W13)</f>
+        <v/>
+      </c>
+      <c r="D35" s="30">
+        <f>IF(LEN(detail!Q13)&lt;1,"",detail!Q13)</f>
+        <v/>
+      </c>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE13)&lt;1,"",detail!AE13), 0) &amp; IF(detail!AF13 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G35" s="30">
+        <f>IF(LEN(detail!AA13)&lt;1,"",detail!AB13)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="18">
-        <f>IF(LEN(detail!K16)&lt;1,"",detail!K16)</f>
-        <v/>
-      </c>
-      <c r="C36" s="18">
-        <f>IF(LEN(detail!S16)&lt;1,"", detail!S16)</f>
-        <v/>
-      </c>
-      <c r="D36" s="26">
-        <f>IF(LEN(detail!M16)&lt;1,"",detail!M16)</f>
-        <v/>
-      </c>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="11">
-        <f>DOLLAR(IF(LEN(detail!X16)&lt;1,"",detail!X16), 0) &amp; IF(detail!Y16 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G36" s="26">
-        <f>IF(LEN(detail!W16)&lt;1,"",detail!W16)</f>
+      <c r="B36" s="14">
+        <f>IF(LEN(detail!O14)&lt;1,"",detail!O14)</f>
+        <v/>
+      </c>
+      <c r="C36" s="14">
+        <f>IF(LEN(detail!W14)&lt;1,"", detail!W14)</f>
+        <v/>
+      </c>
+      <c r="D36" s="30">
+        <f>IF(LEN(detail!Q14)&lt;1,"",detail!Q14)</f>
+        <v/>
+      </c>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE14)&lt;1,"",detail!AE14), 0) &amp; IF(detail!AF14 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G36" s="30">
+        <f>IF(LEN(detail!AA14)&lt;1,"",detail!AB14)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="18">
-        <f>IF(LEN(detail!K17)&lt;1,"",detail!K17)</f>
-        <v/>
-      </c>
-      <c r="C37" s="18">
-        <f>IF(LEN(detail!S17)&lt;1,"", detail!S17)</f>
-        <v/>
-      </c>
-      <c r="D37" s="26">
-        <f>IF(LEN(detail!M17)&lt;1,"",detail!M17)</f>
-        <v/>
-      </c>
-      <c r="E37" s="27" t="n"/>
-      <c r="F37" s="11">
-        <f>DOLLAR(IF(LEN(detail!X17)&lt;1,"",detail!X17), 0) &amp; IF(detail!Y17 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G37" s="26">
-        <f>IF(LEN(detail!W17)&lt;1,"",detail!W17)</f>
+      <c r="B37" s="14">
+        <f>IF(LEN(detail!O15)&lt;1,"",detail!O15)</f>
+        <v/>
+      </c>
+      <c r="C37" s="14">
+        <f>IF(LEN(detail!W15)&lt;1,"", detail!W15)</f>
+        <v/>
+      </c>
+      <c r="D37" s="30">
+        <f>IF(LEN(detail!Q15)&lt;1,"",detail!Q15)</f>
+        <v/>
+      </c>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE15)&lt;1,"",detail!AE15), 0) &amp; IF(detail!AF15 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G37" s="30">
+        <f>IF(LEN(detail!AA15)&lt;1,"",detail!AB15)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="18">
-        <f>IF(LEN(detail!K18)&lt;1,"",detail!K18)</f>
-        <v/>
-      </c>
-      <c r="C38" s="18">
-        <f>IF(LEN(detail!S18)&lt;1,"", detail!S18)</f>
-        <v/>
-      </c>
-      <c r="D38" s="26">
-        <f>IF(LEN(detail!M18)&lt;1,"",detail!M18)</f>
-        <v/>
-      </c>
-      <c r="E38" s="27" t="n"/>
-      <c r="F38" s="11">
-        <f>DOLLAR(IF(LEN(detail!X18)&lt;1,"",detail!X18), 0) &amp; IF(detail!Y18 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G38" s="26">
-        <f>IF(LEN(detail!W18)&lt;1,"",detail!W18)</f>
+      <c r="B38" s="14">
+        <f>IF(LEN(detail!O16)&lt;1,"",detail!O16)</f>
+        <v/>
+      </c>
+      <c r="C38" s="14">
+        <f>IF(LEN(detail!W16)&lt;1,"", detail!W16)</f>
+        <v/>
+      </c>
+      <c r="D38" s="30">
+        <f>IF(LEN(detail!Q16)&lt;1,"",detail!Q16)</f>
+        <v/>
+      </c>
+      <c r="E38" s="31" t="n"/>
+      <c r="F38" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE16)&lt;1,"",detail!AE16), 0) &amp; IF(detail!AF16 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G38" s="30">
+        <f>IF(LEN(detail!AA16)&lt;1,"",detail!AB16)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="18">
-        <f>IF(LEN(detail!K19)&lt;1,"",detail!K19)</f>
-        <v/>
-      </c>
-      <c r="C39" s="18">
-        <f>IF(LEN(detail!S19)&lt;1,"", detail!S19)</f>
-        <v/>
-      </c>
-      <c r="D39" s="26">
-        <f>IF(LEN(detail!M19)&lt;1,"",detail!M19)</f>
-        <v/>
-      </c>
-      <c r="E39" s="27" t="n"/>
-      <c r="F39" s="11">
-        <f>DOLLAR(IF(LEN(detail!X19)&lt;1,"",detail!X19), 0) &amp; IF(detail!Y19 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G39" s="26">
-        <f>IF(LEN(detail!W19)&lt;1,"",detail!W19)</f>
+      <c r="B39" s="14">
+        <f>IF(LEN(detail!O17)&lt;1,"",detail!O17)</f>
+        <v/>
+      </c>
+      <c r="C39" s="14">
+        <f>IF(LEN(detail!W17)&lt;1,"", detail!W17)</f>
+        <v/>
+      </c>
+      <c r="D39" s="30">
+        <f>IF(LEN(detail!Q17)&lt;1,"",detail!Q17)</f>
+        <v/>
+      </c>
+      <c r="E39" s="31" t="n"/>
+      <c r="F39" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE17)&lt;1,"",detail!AE17), 0) &amp; IF(detail!AF17 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G39" s="30">
+        <f>IF(LEN(detail!AA17)&lt;1,"",detail!AB17)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="18">
-        <f>IF(LEN(detail!K20)&lt;1,"",detail!K20)</f>
-        <v/>
-      </c>
-      <c r="C40" s="18">
-        <f>IF(LEN(detail!S20)&lt;1,"", detail!S20)</f>
-        <v/>
-      </c>
-      <c r="D40" s="26">
-        <f>IF(LEN(detail!M20)&lt;1,"",detail!M20)</f>
-        <v/>
-      </c>
-      <c r="E40" s="27" t="n"/>
-      <c r="F40" s="11">
-        <f>DOLLAR(IF(LEN(detail!X20)&lt;1,"",detail!X20), 0) &amp; IF(detail!Y20 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G40" s="26">
-        <f>IF(LEN(detail!W20)&lt;1,"",detail!W20)</f>
+      <c r="B40" s="14">
+        <f>IF(LEN(detail!O18)&lt;1,"",detail!O18)</f>
+        <v/>
+      </c>
+      <c r="C40" s="14">
+        <f>IF(LEN(detail!W18)&lt;1,"", detail!W18)</f>
+        <v/>
+      </c>
+      <c r="D40" s="30">
+        <f>IF(LEN(detail!Q18)&lt;1,"",detail!Q18)</f>
+        <v/>
+      </c>
+      <c r="E40" s="31" t="n"/>
+      <c r="F40" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE18)&lt;1,"",detail!AE18), 0) &amp; IF(detail!AF18 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G40" s="30">
+        <f>IF(LEN(detail!AA18)&lt;1,"",detail!AB18)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="18">
-        <f>IF(LEN(detail!K21)&lt;1,"",detail!K21)</f>
-        <v/>
-      </c>
-      <c r="C41" s="18">
-        <f>IF(LEN(detail!S21)&lt;1,"", detail!S21)</f>
-        <v/>
-      </c>
-      <c r="D41" s="26">
-        <f>IF(LEN(detail!M21)&lt;1,"",detail!M21)</f>
-        <v/>
-      </c>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="11">
-        <f>DOLLAR(IF(LEN(detail!X21)&lt;1,"",detail!X21), 0) &amp; IF(detail!Y21 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G41" s="26">
-        <f>IF(LEN(detail!W21)&lt;1,"",detail!W21)</f>
+      <c r="B41" s="14">
+        <f>IF(LEN(detail!O19)&lt;1,"",detail!O19)</f>
+        <v/>
+      </c>
+      <c r="C41" s="14">
+        <f>IF(LEN(detail!W19)&lt;1,"", detail!W19)</f>
+        <v/>
+      </c>
+      <c r="D41" s="30">
+        <f>IF(LEN(detail!Q19)&lt;1,"",detail!Q19)</f>
+        <v/>
+      </c>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE19)&lt;1,"",detail!AE19), 0) &amp; IF(detail!AF19 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G41" s="30">
+        <f>IF(LEN(detail!AA19)&lt;1,"",detail!AB19)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="18">
-        <f>IF(LEN(detail!K22)&lt;1,"",detail!K22)</f>
-        <v/>
-      </c>
-      <c r="C42" s="18">
-        <f>IF(LEN(detail!S22)&lt;1,"", detail!S22)</f>
-        <v/>
-      </c>
-      <c r="D42" s="26">
-        <f>IF(LEN(detail!M22)&lt;1,"",detail!M22)</f>
-        <v/>
-      </c>
-      <c r="E42" s="27" t="n"/>
-      <c r="F42" s="11">
-        <f>DOLLAR(IF(LEN(detail!X22)&lt;1,"",detail!X22), 0) &amp; IF(detail!Y22 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G42" s="26">
-        <f>IF(LEN(detail!W22)&lt;1,"",detail!W22)</f>
+      <c r="B42" s="14">
+        <f>IF(LEN(detail!O20)&lt;1,"",detail!O20)</f>
+        <v/>
+      </c>
+      <c r="C42" s="14">
+        <f>IF(LEN(detail!W20)&lt;1,"", detail!W20)</f>
+        <v/>
+      </c>
+      <c r="D42" s="30">
+        <f>IF(LEN(detail!Q20)&lt;1,"",detail!Q20)</f>
+        <v/>
+      </c>
+      <c r="E42" s="31" t="n"/>
+      <c r="F42" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE20)&lt;1,"",detail!AE20), 0) &amp; IF(detail!AF20 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G42" s="30">
+        <f>IF(LEN(detail!AA20)&lt;1,"",detail!AB20)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="18">
-        <f>IF(LEN(detail!K23)&lt;1,"",detail!K23)</f>
-        <v/>
-      </c>
-      <c r="C43" s="18">
-        <f>IF(LEN(detail!S23)&lt;1,"", detail!S23)</f>
-        <v/>
-      </c>
-      <c r="D43" s="26">
-        <f>IF(LEN(detail!M23)&lt;1,"",detail!M23)</f>
-        <v/>
-      </c>
-      <c r="E43" s="27" t="n"/>
-      <c r="F43" s="11">
-        <f>DOLLAR(IF(LEN(detail!X23)&lt;1,"",detail!X23), 0) &amp; IF(detail!Y23 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G43" s="26">
-        <f>IF(LEN(detail!W23)&lt;1,"",detail!W23)</f>
+      <c r="B43" s="14">
+        <f>IF(LEN(detail!O21)&lt;1,"",detail!O21)</f>
+        <v/>
+      </c>
+      <c r="C43" s="14">
+        <f>IF(LEN(detail!W21)&lt;1,"", detail!W21)</f>
+        <v/>
+      </c>
+      <c r="D43" s="30">
+        <f>IF(LEN(detail!Q21)&lt;1,"",detail!Q21)</f>
+        <v/>
+      </c>
+      <c r="E43" s="31" t="n"/>
+      <c r="F43" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE21)&lt;1,"",detail!AE21), 0) &amp; IF(detail!AF21 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G43" s="30">
+        <f>IF(LEN(detail!AA21)&lt;1,"",detail!AB21)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="18">
-        <f>IF(LEN(detail!K24)&lt;1,"",detail!K24)</f>
-        <v/>
-      </c>
-      <c r="C44" s="18">
-        <f>IF(LEN(detail!S24)&lt;1,"", detail!S24)</f>
-        <v/>
-      </c>
-      <c r="D44" s="26">
-        <f>IF(LEN(detail!M24)&lt;1,"",detail!M24)</f>
-        <v/>
-      </c>
-      <c r="E44" s="27" t="n"/>
-      <c r="F44" s="11">
-        <f>DOLLAR(IF(LEN(detail!X24)&lt;1,"",detail!X24), 0) &amp; IF(detail!Y24 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G44" s="26">
-        <f>IF(LEN(detail!W24)&lt;1,"",detail!W24)</f>
+      <c r="B44" s="14">
+        <f>IF(LEN(detail!O22)&lt;1,"",detail!O22)</f>
+        <v/>
+      </c>
+      <c r="C44" s="14">
+        <f>IF(LEN(detail!W22)&lt;1,"", detail!W22)</f>
+        <v/>
+      </c>
+      <c r="D44" s="30">
+        <f>IF(LEN(detail!Q22)&lt;1,"",detail!Q22)</f>
+        <v/>
+      </c>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE22)&lt;1,"",detail!AE22), 0) &amp; IF(detail!AF22 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G44" s="30">
+        <f>IF(LEN(detail!AA22)&lt;1,"",detail!AB22)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="1" t="inlineStr">
+      <c r="B45" s="14">
+        <f>IF(LEN(detail!O23)&lt;1,"",detail!O23)</f>
+        <v/>
+      </c>
+      <c r="C45" s="14">
+        <f>IF(LEN(detail!W23)&lt;1,"", detail!W23)</f>
+        <v/>
+      </c>
+      <c r="D45" s="30">
+        <f>IF(LEN(detail!Q23)&lt;1,"",detail!Q23)</f>
+        <v/>
+      </c>
+      <c r="E45" s="31" t="n"/>
+      <c r="F45" s="9">
+        <f>DOLLAR(IF(LEN(detail!AE23)&lt;1,"",detail!AE23), 0) &amp; IF(detail!AF23 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G45" s="30">
+        <f>IF(LEN(detail!AA23)&lt;1,"",detail!AB23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="1" t="inlineStr">
         <is>
           <t>* An asterisk denotes that the opp includes a rebate</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="36">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D22:E22"/>
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E19:F19"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="E13:F13"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B20:G20"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="E11:F11"/>
@@ -1801,20 +1903,21 @@
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="D33:E33"/>
     <mergeCell ref="D42:E42"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D33:E33"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D35:E35"/>
   </mergeCells>
-  <conditionalFormatting sqref="B22:D44 F22:G44">
+  <conditionalFormatting sqref="B24:D45 F24:G45">
     <cfRule type="containsErrors" priority="1" dxfId="0">
-      <formula>ISERROR(B22)</formula>
+      <formula>ISERROR(B24)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1829,46 +1932,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>YYYYMM</t>
         </is>
       </c>
-      <c r="B1" s="42" t="inlineStr">
+      <c r="B1" s="47" t="inlineStr">
         <is>
           <t>EID</t>
         </is>
       </c>
-      <c r="C1" s="42" t="inlineStr">
+      <c r="C1" s="47" t="inlineStr">
         <is>
           <t>YYYYQQ</t>
         </is>
       </c>
-      <c r="D1" s="42" t="inlineStr">
+      <c r="D1" s="47" t="inlineStr">
         <is>
           <t>ROLE</t>
         </is>
       </c>
-      <c r="E1" s="42" t="inlineStr">
+      <c r="E1" s="47" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="F1" s="42" t="inlineStr">
+      <c r="F1" s="47" t="inlineStr">
         <is>
           <t>VALUE</t>
         </is>
       </c>
-      <c r="G1" s="42" t="inlineStr">
+      <c r="G1" s="47" t="inlineStr">
         <is>
           <t>CATEGORY</t>
         </is>
       </c>
-      <c r="H1" s="42" t="inlineStr">
+      <c r="H1" s="47" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1877,17 +1980,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1912,17 +2015,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1947,17 +2050,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1982,17 +2085,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2017,17 +2120,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2052,17 +2155,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2080,24 +2183,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CS_DEDUCTION</t>
+          <t>IMPLANT_ACCEL_TRUE_UP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2115,24 +2218,24 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>TTL_PO</t>
+          <t>PROGRAM_ACCEL_PO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2150,24 +2253,24 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>GUR_AMT</t>
+          <t>CS_DEDUCTION</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2185,24 +2288,24 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PO_AMT</t>
+          <t>TTL_PO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2216,28 +2319,28 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>12500</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>IMPLANT_UNITS</t>
+          <t>GUR_AMT</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2251,28 +2354,28 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>12500</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>REVENUE_UNITS</t>
+          <t>PO_AMT</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025_01</t>
+          <t>2025_08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025_Q1</t>
+          <t>2025_Q3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2286,9 +2389,149 @@
         </is>
       </c>
       <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>IMPLANT_UNITS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ycruea@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>0</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>REVENUE_UNITS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ycruea@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>QTD_SALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ycruea@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>QTD_IMPL_REV_RATIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ycruea@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>YTD_PO</t>
         </is>
@@ -2320,7 +2563,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Wade Steinhoff</t>
+          <t>Y-Lan Cruea</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2575,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>wsteinhoff@cvrx.com</t>
+          <t>ycruea@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2599,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SACRAMENTO (STEINHOFF)</t>
+          <t>ORANGE COUNTY (CRUEA)</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2623,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>August</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2634,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>151288.0362</v>
+        <v>174570.6546</v>
       </c>
     </row>
     <row r="8">
@@ -2401,7 +2644,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>168097.818</v>
+        <v>226295.2929</v>
       </c>
     </row>
     <row r="21" ht="15.95" customHeight="1"/>
@@ -2419,211 +2662,246 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO1"/>
+  <dimension ref="A1:AV1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>SALES_CREDIT_REP_EMAIL</t>
         </is>
       </c>
-      <c r="B1" s="42" t="inlineStr">
+      <c r="B1" s="47" t="inlineStr">
         <is>
           <t>NAME_REP</t>
         </is>
       </c>
-      <c r="C1" s="42" t="inlineStr">
+      <c r="C1" s="47" t="inlineStr">
+        <is>
+          <t>COVERAGE_TYPE</t>
+        </is>
+      </c>
+      <c r="D1" s="47" t="inlineStr">
+        <is>
+          <t>REP_TERR_ID</t>
+        </is>
+      </c>
+      <c r="E1" s="47" t="inlineStr">
+        <is>
+          <t>ZIP_TERR_ID</t>
+        </is>
+      </c>
+      <c r="F1" s="47" t="inlineStr">
         <is>
           <t>REGION_NM</t>
         </is>
       </c>
-      <c r="D1" s="42" t="inlineStr">
+      <c r="G1" s="47" t="inlineStr">
         <is>
           <t>REGION_ID</t>
         </is>
       </c>
-      <c r="E1" s="42" t="inlineStr">
+      <c r="H1" s="47" t="inlineStr">
         <is>
           <t>CLOSEDATE</t>
         </is>
       </c>
-      <c r="F1" s="42" t="inlineStr">
+      <c r="I1" s="47" t="inlineStr">
         <is>
           <t>CLOSE_YYYYMM</t>
         </is>
       </c>
-      <c r="G1" s="42" t="inlineStr">
+      <c r="J1" s="47" t="inlineStr">
         <is>
           <t>CLOSE_YYYYQQ</t>
         </is>
       </c>
-      <c r="H1" s="42" t="inlineStr">
+      <c r="K1" s="47" t="inlineStr">
         <is>
           <t>IMPLANTED_DT</t>
         </is>
       </c>
-      <c r="I1" s="42" t="inlineStr">
+      <c r="L1" s="47" t="inlineStr">
         <is>
           <t>IMPLANTED_YYYYMM</t>
         </is>
       </c>
-      <c r="J1" s="42" t="inlineStr">
+      <c r="M1" s="47" t="inlineStr">
         <is>
           <t>IMPLANTED_YYYYQQ</t>
         </is>
       </c>
-      <c r="K1" s="42" t="inlineStr">
+      <c r="N1" s="47" t="inlineStr">
+        <is>
+          <t>DHC_IDN_NAME__C</t>
+        </is>
+      </c>
+      <c r="O1" s="47" t="inlineStr">
         <is>
           <t>ACCOUNT_INDICATION__C</t>
         </is>
       </c>
-      <c r="L1" s="42" t="inlineStr">
+      <c r="P1" s="47" t="inlineStr">
         <is>
           <t>ACT_ID</t>
         </is>
       </c>
-      <c r="M1" s="42" t="inlineStr">
+      <c r="Q1" s="47" t="inlineStr">
         <is>
           <t>OPP_NAME</t>
         </is>
       </c>
-      <c r="N1" s="42" t="inlineStr">
+      <c r="R1" s="47" t="inlineStr">
         <is>
           <t>OPP_ID</t>
         </is>
       </c>
-      <c r="O1" s="42" t="inlineStr">
+      <c r="S1" s="47" t="inlineStr">
         <is>
           <t>OPP_OWNER_EMAIL</t>
         </is>
       </c>
-      <c r="P1" s="42" t="inlineStr">
+      <c r="T1" s="47" t="inlineStr">
         <is>
           <t>PHYSICIAN</t>
         </is>
       </c>
-      <c r="Q1" s="42" t="inlineStr">
+      <c r="U1" s="47" t="inlineStr">
         <is>
           <t>PHYSICIAN_ID</t>
         </is>
       </c>
-      <c r="R1" s="42" t="inlineStr">
+      <c r="V1" s="47" t="inlineStr">
         <is>
           <t>INDICATION_FOR_USE__C</t>
         </is>
       </c>
-      <c r="S1" s="42" t="inlineStr">
+      <c r="W1" s="47" t="inlineStr">
         <is>
           <t>REASON_FOR_IMPLANT__C</t>
         </is>
       </c>
-      <c r="T1" s="42" t="inlineStr">
+      <c r="X1" s="47" t="inlineStr">
         <is>
           <t>STAGENAME</t>
         </is>
       </c>
-      <c r="U1" s="42" t="inlineStr">
+      <c r="Y1" s="47" t="inlineStr">
         <is>
           <t>ISIMPL</t>
         </is>
       </c>
-      <c r="V1" s="42" t="inlineStr">
+      <c r="Z1" s="47" t="inlineStr">
         <is>
           <t>IMPLANT_UNITS</t>
         </is>
       </c>
-      <c r="W1" s="42" t="inlineStr">
+      <c r="AA1" s="47" t="inlineStr">
+        <is>
+          <t>IMPLANT_UNITS_FOR_RATIO</t>
+        </is>
+      </c>
+      <c r="AB1" s="47" t="inlineStr">
         <is>
           <t>REVENUE_UNITS</t>
         </is>
       </c>
-      <c r="X1" s="42" t="inlineStr">
+      <c r="AC1" s="47" t="inlineStr">
+        <is>
+          <t>REV_UNITS_FOR_RATIO</t>
+        </is>
+      </c>
+      <c r="AD1" s="47" t="inlineStr">
         <is>
           <t>SALES</t>
         </is>
       </c>
-      <c r="Y1" s="42" t="inlineStr">
+      <c r="AE1" s="47" t="inlineStr">
+        <is>
+          <t>SALES_COMMISSIONABLE</t>
+        </is>
+      </c>
+      <c r="AF1" s="47" t="inlineStr">
         <is>
           <t>REBATE?</t>
         </is>
       </c>
-      <c r="Z1" s="42" t="inlineStr">
+      <c r="AG1" s="47" t="inlineStr">
         <is>
           <t>ASP</t>
         </is>
       </c>
-      <c r="AA1" s="42" t="inlineStr">
+      <c r="AH1" s="47" t="inlineStr">
         <is>
           <t>THRESHOLD</t>
         </is>
       </c>
-      <c r="AB1" s="42" t="inlineStr">
+      <c r="AI1" s="47" t="inlineStr">
         <is>
           <t>PLAN</t>
         </is>
       </c>
-      <c r="AC1" s="42" t="inlineStr">
-        <is>
-          <t>QTD_SALES</t>
-        </is>
-      </c>
-      <c r="AD1" s="42" t="inlineStr">
+      <c r="AJ1" s="47" t="inlineStr">
+        <is>
+          <t>QTD_SALES_COMISSIONABLE</t>
+        </is>
+      </c>
+      <c r="AK1" s="47" t="inlineStr">
         <is>
           <t>QTD_IMPLANT_UNITS</t>
         </is>
       </c>
-      <c r="AE1" s="42" t="inlineStr">
+      <c r="AL1" s="47" t="inlineStr">
         <is>
           <t>QTD_REVENUE_UNITS</t>
         </is>
       </c>
-      <c r="AF1" s="42" t="inlineStr">
+      <c r="AM1" s="47" t="inlineStr">
         <is>
           <t>CS_PO_EMAIL</t>
         </is>
       </c>
-      <c r="AG1" s="42" t="inlineStr">
+      <c r="AN1" s="47" t="inlineStr">
         <is>
           <t>CS_PO_$</t>
         </is>
       </c>
-      <c r="AH1" s="42" t="inlineStr">
+      <c r="AO1" s="47" t="inlineStr">
         <is>
           <t>CS_PO_%</t>
         </is>
       </c>
-      <c r="AI1" s="42" t="inlineStr">
+      <c r="AP1" s="47" t="inlineStr">
         <is>
           <t>CS_PO_TYPE</t>
         </is>
       </c>
-      <c r="AJ1" s="42" t="inlineStr">
+      <c r="AQ1" s="47" t="inlineStr">
         <is>
           <t>CS_PO_YYYYMM</t>
         </is>
       </c>
-      <c r="AK1" s="42" t="inlineStr">
+      <c r="AR1" s="47" t="inlineStr">
         <is>
           <t>L1_REV</t>
         </is>
       </c>
-      <c r="AL1" s="42" t="inlineStr">
+      <c r="AS1" s="47" t="inlineStr">
         <is>
           <t>L2_REV</t>
         </is>
       </c>
-      <c r="AM1" s="42" t="inlineStr">
+      <c r="AT1" s="47" t="inlineStr">
         <is>
           <t>QTD_IMPL_REV_RATIO</t>
         </is>
       </c>
-      <c r="AN1" s="42" t="inlineStr">
+      <c r="AU1" s="47" t="inlineStr">
         <is>
           <t>L1_PO</t>
         </is>
       </c>
-      <c r="AO1" s="42" t="inlineStr">
+      <c r="AV1" s="47" t="inlineStr">
         <is>
           <t>L2_PO</t>
         </is>

</xml_diff>

<commit_message>
update VBA so you no longer need to edit export filepath each month
</commit_message>
<xml_diff>
--- a/Excel Files/COMP_STATEMENT.xlsx
+++ b/Excel Files/COMP_STATEMENT.xlsx
@@ -1106,6 +1106,10 @@
         <f>info!B6 &amp; " 2025"</f>
         <v/>
       </c>
+      <c r="C6" s="5">
+        <f>_xlfn.CONCAT(TEXT(B6,"YYYY"), "_", TEXT(B6,"MM"))</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="3.95" customHeight="1"/>
     <row r="8" ht="3.95" customHeight="1" thickBot="1"/>
@@ -1884,15 +1888,14 @@
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D31:E31"/>
     <mergeCell ref="E17:F17"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="D26:E26"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="D43:E43"/>
@@ -1902,16 +1905,17 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D24:E24"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D24:E24"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D42:E42"/>
     <mergeCell ref="D29:E29"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="D38:E38"/>
-    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D35:E35"/>
   </mergeCells>
@@ -1985,7 +1989,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2004,7 +2008,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2020,7 +2024,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2039,7 +2043,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2055,7 +2059,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2074,7 +2078,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>4725</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2090,7 +2094,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2125,7 +2129,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2160,7 +2164,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2195,7 +2199,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2230,7 +2234,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2265,7 +2269,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2284,7 +2288,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>4725</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2300,7 +2304,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2319,7 +2323,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>12500</v>
+        <v>18333.33</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2335,7 +2339,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2354,7 +2358,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>12500</v>
+        <v>18333.33</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2370,7 +2374,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2405,7 +2409,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2424,7 +2428,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -2440,7 +2444,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2459,7 +2463,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>31500</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -2475,7 +2479,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2510,7 +2514,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2529,7 +2533,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>25000</v>
+        <v>82500</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2563,7 +2567,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Y-Lan Cruea</t>
+          <t>Adam Benwitz</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2579,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>abenwitz@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2591,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mbrown@cvrx.com</t>
+          <t>jhorky@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2603,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ORANGE COUNTY (CRUEA)</t>
+          <t>CHICAGO II (BENWITZ)</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV1"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2907,6 +2911,174 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>abenwitz@cvrx.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Adam Benwitz</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TERR_92</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TERR_92</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>MIDWEST</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>RE_01</t>
+        </is>
+      </c>
+      <c r="H2" s="49" t="n">
+        <v>45883</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2025_08</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2025_Q3</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>NorthShore - Edward-Elmhurst Health</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Glenbrook Northshore Hospital</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0010g00001m5aQmAAI</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ORD02 026868</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>006UY00000OYbP7YAL</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>abenwitz@cvrx.com</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Heart Failure - Reduced Ejection Fraction</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Replacement</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Revenue Recognized</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>174570.6546</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>226295.2929</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>4725</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
new statements for ATMs
</commit_message>
<xml_diff>
--- a/Excel Files/COMP_STATEMENT.xlsx
+++ b/Excel Files/COMP_STATEMENT.xlsx
@@ -18,13 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,8 +82,15 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -109,8 +115,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="33">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -461,6 +473,30 @@
     </border>
     <border>
       <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top style="hair">
         <color indexed="64"/>
@@ -474,35 +510,6 @@
         <color indexed="64"/>
       </right>
       <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="double">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="double">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -525,6 +532,35 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="double">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -534,7 +570,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -596,46 +632,60 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1034,7 +1084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K46"/>
+  <dimension ref="A2:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="0.7109375" customWidth="1" style="1" min="1" max="1"/>
@@ -1081,147 +1131,160 @@
     <row r="7" ht="3.95" customHeight="1"/>
     <row r="8" ht="3.95" customHeight="1" thickBot="1"/>
     <row r="9">
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="34" t="inlineStr">
         <is>
           <t>Sales Performance</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n"/>
+      <c r="C9" s="36" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="E9" s="34" t="inlineStr">
         <is>
           <t>Final Payment</t>
         </is>
       </c>
-      <c r="F9" s="43" t="n"/>
-      <c r="G9" s="29" t="n"/>
+      <c r="F9" s="35" t="n"/>
+      <c r="G9" s="36" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>ATM Account Sales</t>
+        </is>
+      </c>
+      <c r="C10" s="50">
+        <f>_xlfn.XLOOKUP("ATM_ACCOUNT_REV", payout!G:G,payout!F:F)</f>
+        <v/>
+      </c>
+      <c r="D10" s="28">
+        <f>IF(G10&gt;0, 1, 0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>ATM Account Payout</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="49">
+        <f>_xlfn.XLOOKUP("ATM_ACCOUNT_PO", payout!G:G,payout!F:F)</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>C10*0.15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Level 1 Sales</t>
         </is>
       </c>
-      <c r="C10" s="19">
+      <c r="C11" s="19">
         <f>_xlfn.XLOOKUP("L1_REV", payout!$G:$G, payout!$F:$F)</f>
         <v/>
       </c>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="38" t="inlineStr">
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="29" t="inlineStr">
         <is>
           <t>Level 1 Payout</t>
         </is>
       </c>
-      <c r="F10" s="31" t="n"/>
-      <c r="G10" s="6">
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="6">
         <f>_xlfn.XLOOKUP("L1_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
-      <c r="K10" s="15">
-        <f>C10*0.15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="38" t="inlineStr">
+      <c r="K11" s="15">
+        <f>C11*0.15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Level 2 Sales</t>
         </is>
       </c>
-      <c r="C11" s="21">
+      <c r="C12" s="21">
         <f>_xlfn.XLOOKUP("L2_REV", payout!$G:$G, payout!$F:$F)</f>
         <v/>
       </c>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="38" t="inlineStr">
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>Level 2 Payout</t>
         </is>
       </c>
-      <c r="F11" s="31" t="n"/>
-      <c r="G11" s="12">
-        <f>(_xlfn.XLOOKUP("L2_PO",payout!G:G,payout!F:F))</f>
-        <v/>
-      </c>
-      <c r="K11" s="15">
-        <f>C11*0.2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B12" s="10" t="inlineStr">
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="12">
+        <f>_xlfn.XLOOKUP("L2_PO",payout!G:G,payout!F:F)</f>
+        <v/>
+      </c>
+      <c r="K12" s="15">
+        <f>C12*0.2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Total Sales</t>
         </is>
       </c>
-      <c r="C12" s="20">
-        <f>SUM(C10:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="35" t="inlineStr">
+      <c r="C13" s="20">
+        <f>SUM(C10:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="43" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="F12" s="36" t="n"/>
-      <c r="G12" s="13">
-        <f>SUM(G10:G11)</f>
-        <v/>
-      </c>
-      <c r="K12" s="15" t="n"/>
-    </row>
-    <row r="13" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B13" s="16" t="inlineStr">
+      <c r="F13" s="44" t="n"/>
+      <c r="G13" s="13">
+        <f>SUM(G10:G12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="15" t="n"/>
+    </row>
+    <row r="14" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>QTD Sales</t>
         </is>
       </c>
-      <c r="C13" s="18">
+      <c r="C14" s="18">
         <f>_xlfn.IFNA(_xlfn.XLOOKUP("QTD_SALES", payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="41" t="inlineStr">
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="37" t="inlineStr">
         <is>
           <t>Adjustments</t>
         </is>
       </c>
-      <c r="F13" s="42" t="n"/>
-      <c r="G13" s="11">
+      <c r="F14" s="38" t="n"/>
+      <c r="G14" s="11">
         <f>_xlfn.IFNA(_xlfn.XLOOKUP("ADJUSTMENTS", payout!G:G,payout!F:F), 0) + _xlfn.IFNA(_xlfn.XLOOKUP("T-SPLIT", payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="D14" s="5" t="n">
+    <row r="15">
+      <c r="D15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="44" t="inlineStr">
+      <c r="E15" s="45" t="inlineStr">
         <is>
           <t>CPAS Payout</t>
         </is>
       </c>
-      <c r="F14" s="31" t="n"/>
-      <c r="G14" s="11">
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="11">
         <f>IFERROR(_xlfn.XLOOKUP("CPAS_PO", payout!G:G,payout!F:F), 0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="16.5" customHeight="1">
-      <c r="D15" s="5">
-        <f>IF(G15&gt;0, 1, 0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="32" t="inlineStr">
-        <is>
-          <t>Program Accel</t>
-        </is>
-      </c>
-      <c r="F15" s="31" t="n"/>
-      <c r="G15" s="11">
-        <f>IFERROR(_xlfn.XLOOKUP("PROGRAM_ACCEL_PO",payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
@@ -1230,638 +1293,658 @@
         <f>IF(G16&gt;0, 1, 0)</f>
         <v/>
       </c>
-      <c r="E16" s="32" t="inlineStr">
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>Program Accel</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="n"/>
+      <c r="G16" s="11">
+        <f>IFERROR(_xlfn.XLOOKUP("PROGRAM_ACCEL_PO",payout!G:G,payout!F:F), 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1">
+      <c r="D17" s="5">
+        <f>IF(G17&gt;0, 1, 0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>Implant Ratio Accel</t>
         </is>
       </c>
-      <c r="F16" s="31" t="n"/>
-      <c r="G16" s="11">
+      <c r="F17" s="30" t="n"/>
+      <c r="G17" s="11">
         <f>IFERROR(_xlfn.XLOOKUP("IMPLANT_ACCEL_TRUE_UP",payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" thickBot="1">
-      <c r="D17" s="5">
-        <f>IF(G17&gt;0, IF(G17&gt;IFERROR(_xlfn.XLOOKUP("TTL_PO", payout!G:G,payout!F:F), 0), 1, 0), 0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="45" t="inlineStr">
-        <is>
-          <t>Recoverable Draw</t>
-        </is>
-      </c>
-      <c r="F17" s="46" t="n"/>
-      <c r="G17" s="25">
+    <row r="18" ht="16.5" customHeight="1" thickBot="1">
+      <c r="D18" s="5">
+        <f>IF(G18&gt;0, IF(G18&gt;IFERROR(_xlfn.XLOOKUP("TTL_PO", payout!G:G,payout!F:F), 0), 1, 0), 0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>Minimum Payout</t>
+        </is>
+      </c>
+      <c r="F18" s="48" t="n"/>
+      <c r="G18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP("GUR_AMT",payout!G:G,payout!F:F), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="35" t="inlineStr">
+    <row r="19" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="43" t="inlineStr">
         <is>
           <t>Final Payout</t>
         </is>
       </c>
-      <c r="F18" s="36" t="n"/>
-      <c r="G18" s="26">
+      <c r="F19" s="44" t="n"/>
+      <c r="G19" s="26">
         <f>_xlfn.XLOOKUP("PO_AMT", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
-      <c r="B19" s="22" t="inlineStr">
+    <row r="20" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>Q1 Threshold</t>
         </is>
       </c>
-      <c r="C19" s="23">
+      <c r="C20" s="23">
         <f>info!B7</f>
         <v/>
       </c>
-      <c r="E19" s="39" t="inlineStr">
+      <c r="E20" s="40" t="inlineStr">
         <is>
           <t>YTD Payout</t>
         </is>
       </c>
-      <c r="F19" s="40" t="n"/>
-      <c r="G19" s="17">
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="17">
         <f>_xlfn.XLOOKUP("YTD_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="3.95" customHeight="1"/>
     <row r="21" ht="3.95" customHeight="1"/>
-    <row r="22">
-      <c r="B22" s="33" t="inlineStr">
+    <row r="22" ht="3.95" customHeight="1"/>
+    <row r="23">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Opportunity Detail </t>
         </is>
       </c>
-      <c r="C22" s="34" t="n"/>
-      <c r="D22" s="34" t="n"/>
-      <c r="E22" s="34" t="n"/>
-      <c r="F22" s="34" t="n"/>
-      <c r="G22" s="31" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="37" t="inlineStr">
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="30" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="46" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C23" s="37" t="inlineStr">
+      <c r="C24" s="46" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D23" s="37" t="inlineStr">
+      <c r="D24" s="46" t="inlineStr">
         <is>
           <t>Opp Name</t>
         </is>
       </c>
-      <c r="E23" s="31" t="n"/>
-      <c r="F23" s="37" t="inlineStr">
+      <c r="E24" s="30" t="n"/>
+      <c r="F24" s="46" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="G23" s="37" t="inlineStr">
+      <c r="G24" s="46" t="inlineStr">
         <is>
           <t>Rev Units</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="14">
-        <f>IF(LEN(detail!P2)&lt;1,"",detail!P2)</f>
-        <v/>
-      </c>
-      <c r="C24" s="14">
-        <f>IF(LEN(detail!X2)&lt;1,"", detail!X2)</f>
-        <v/>
-      </c>
-      <c r="D24" s="30">
-        <f>IF(LEN(detail!R2)&lt;1,"",detail!R2)</f>
-        <v/>
-      </c>
-      <c r="E24" s="31" t="n"/>
-      <c r="F24" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF2)&lt;1,"",detail!AF2), 0) &amp; IF(detail!AG2 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G24" s="30">
-        <f>IF(LEN(detail!AC2)&lt;1,"",detail!AC2)</f>
-        <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="14">
-        <f>IF(LEN(detail!P3)&lt;1,"",detail!P3)</f>
+        <f>IF(LEN(detail!P2)&lt;1,"",detail!P2)</f>
         <v/>
       </c>
       <c r="C25" s="14">
-        <f>IF(LEN(detail!X3)&lt;1,"", detail!X3)</f>
-        <v/>
-      </c>
-      <c r="D25" s="30">
-        <f>IF(LEN(detail!R3)&lt;1,"",detail!R3)</f>
-        <v/>
-      </c>
-      <c r="E25" s="31" t="n"/>
+        <f>IF(LEN(detail!X2)&lt;1,"", detail!X2)</f>
+        <v/>
+      </c>
+      <c r="D25" s="31">
+        <f>IF(LEN(detail!R2)&lt;1,"",detail!R2)</f>
+        <v/>
+      </c>
+      <c r="E25" s="30" t="n"/>
       <c r="F25" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF3)&lt;1,"",detail!AF3), 0) &amp; IF(detail!AG3 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G25" s="30">
-        <f>IF(LEN(detail!AC3)&lt;1,"",detail!AC3)</f>
+        <f>DOLLAR(IF(LEN(detail!AF2)&lt;1,"",detail!AF2), 0) &amp; IF(detail!AG2 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>IF(LEN(detail!AC2)&lt;1,"",detail!AC2)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="14">
-        <f>IF(LEN(detail!P4)&lt;1,"",detail!P4)</f>
+        <f>IF(LEN(detail!P3)&lt;1,"",detail!P3)</f>
         <v/>
       </c>
       <c r="C26" s="14">
-        <f>IF(LEN(detail!X4)&lt;1,"", detail!X4)</f>
-        <v/>
-      </c>
-      <c r="D26" s="30">
-        <f>IF(LEN(detail!R4)&lt;1,"",detail!R4)</f>
-        <v/>
-      </c>
-      <c r="E26" s="31" t="n"/>
+        <f>IF(LEN(detail!X3)&lt;1,"", detail!X3)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31">
+        <f>IF(LEN(detail!R3)&lt;1,"",detail!R3)</f>
+        <v/>
+      </c>
+      <c r="E26" s="30" t="n"/>
       <c r="F26" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF4)&lt;1,"",detail!AF4), 0) &amp; IF(detail!AG4 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G26" s="30">
-        <f>IF(LEN(detail!AC4)&lt;1,"",detail!AC4)</f>
+        <f>DOLLAR(IF(LEN(detail!AF3)&lt;1,"",detail!AF3), 0) &amp; IF(detail!AG3 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G26" s="31">
+        <f>IF(LEN(detail!AC3)&lt;1,"",detail!AC3)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="14">
-        <f>IF(LEN(detail!P5)&lt;1,"",detail!P5)</f>
+        <f>IF(LEN(detail!P4)&lt;1,"",detail!P4)</f>
         <v/>
       </c>
       <c r="C27" s="14">
-        <f>IF(LEN(detail!X5)&lt;1,"", detail!X5)</f>
-        <v/>
-      </c>
-      <c r="D27" s="30">
-        <f>IF(LEN(detail!R5)&lt;1,"",detail!R5)</f>
-        <v/>
-      </c>
-      <c r="E27" s="31" t="n"/>
+        <f>IF(LEN(detail!X4)&lt;1,"", detail!X4)</f>
+        <v/>
+      </c>
+      <c r="D27" s="31">
+        <f>IF(LEN(detail!R4)&lt;1,"",detail!R4)</f>
+        <v/>
+      </c>
+      <c r="E27" s="30" t="n"/>
       <c r="F27" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF5)&lt;1,"",detail!AF5), 0) &amp; IF(detail!AG5 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G27" s="30">
-        <f>IF(LEN(detail!AC5)&lt;1,"",detail!AC5)</f>
+        <f>DOLLAR(IF(LEN(detail!AF4)&lt;1,"",detail!AF4), 0) &amp; IF(detail!AG4 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G27" s="31">
+        <f>IF(LEN(detail!AC4)&lt;1,"",detail!AC4)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="14">
-        <f>IF(LEN(detail!P6)&lt;1,"",detail!P6)</f>
+        <f>IF(LEN(detail!P5)&lt;1,"",detail!P5)</f>
         <v/>
       </c>
       <c r="C28" s="14">
-        <f>IF(LEN(detail!X6)&lt;1,"", detail!X6)</f>
-        <v/>
-      </c>
-      <c r="D28" s="30">
-        <f>IF(LEN(detail!R6)&lt;1,"",detail!R6)</f>
-        <v/>
-      </c>
-      <c r="E28" s="31" t="n"/>
+        <f>IF(LEN(detail!X5)&lt;1,"", detail!X5)</f>
+        <v/>
+      </c>
+      <c r="D28" s="31">
+        <f>IF(LEN(detail!R5)&lt;1,"",detail!R5)</f>
+        <v/>
+      </c>
+      <c r="E28" s="30" t="n"/>
       <c r="F28" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF6)&lt;1,"",detail!AF6), 0) &amp; IF(detail!AG6 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G28" s="30">
-        <f>IF(LEN(detail!AC6)&lt;1,"",detail!AC6)</f>
+        <f>DOLLAR(IF(LEN(detail!AF5)&lt;1,"",detail!AF5), 0) &amp; IF(detail!AG5 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G28" s="31">
+        <f>IF(LEN(detail!AC5)&lt;1,"",detail!AC5)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="14">
-        <f>IF(LEN(detail!P7)&lt;1,"",detail!P7)</f>
+        <f>IF(LEN(detail!P6)&lt;1,"",detail!P6)</f>
         <v/>
       </c>
       <c r="C29" s="14">
-        <f>IF(LEN(detail!X7)&lt;1,"", detail!X7)</f>
-        <v/>
-      </c>
-      <c r="D29" s="30">
-        <f>IF(LEN(detail!R7)&lt;1,"",detail!R7)</f>
-        <v/>
-      </c>
-      <c r="E29" s="31" t="n"/>
+        <f>IF(LEN(detail!X6)&lt;1,"", detail!X6)</f>
+        <v/>
+      </c>
+      <c r="D29" s="31">
+        <f>IF(LEN(detail!R6)&lt;1,"",detail!R6)</f>
+        <v/>
+      </c>
+      <c r="E29" s="30" t="n"/>
       <c r="F29" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF7)&lt;1,"",detail!AF7), 0) &amp; IF(detail!AG7 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G29" s="30">
-        <f>IF(LEN(detail!AC7)&lt;1,"",detail!AC7)</f>
+        <f>DOLLAR(IF(LEN(detail!AF6)&lt;1,"",detail!AF6), 0) &amp; IF(detail!AG6 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G29" s="31">
+        <f>IF(LEN(detail!AC6)&lt;1,"",detail!AC6)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="14">
-        <f>IF(LEN(detail!P8)&lt;1,"",detail!P8)</f>
+        <f>IF(LEN(detail!P7)&lt;1,"",detail!P7)</f>
         <v/>
       </c>
       <c r="C30" s="14">
-        <f>IF(LEN(detail!X8)&lt;1,"", detail!X8)</f>
-        <v/>
-      </c>
-      <c r="D30" s="30">
-        <f>IF(LEN(detail!R8)&lt;1,"",detail!R8)</f>
-        <v/>
-      </c>
-      <c r="E30" s="31" t="n"/>
+        <f>IF(LEN(detail!X7)&lt;1,"", detail!X7)</f>
+        <v/>
+      </c>
+      <c r="D30" s="31">
+        <f>IF(LEN(detail!R7)&lt;1,"",detail!R7)</f>
+        <v/>
+      </c>
+      <c r="E30" s="30" t="n"/>
       <c r="F30" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF8)&lt;1,"",detail!AF8), 0) &amp; IF(detail!AG8 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G30" s="30">
-        <f>IF(LEN(detail!AC8)&lt;1,"",detail!AC8)</f>
+        <f>DOLLAR(IF(LEN(detail!AF7)&lt;1,"",detail!AF7), 0) &amp; IF(detail!AG7 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G30" s="31">
+        <f>IF(LEN(detail!AC7)&lt;1,"",detail!AC7)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="14">
-        <f>IF(LEN(detail!P9)&lt;1,"",detail!P9)</f>
+        <f>IF(LEN(detail!P8)&lt;1,"",detail!P8)</f>
         <v/>
       </c>
       <c r="C31" s="14">
-        <f>IF(LEN(detail!X9)&lt;1,"", detail!X9)</f>
-        <v/>
-      </c>
-      <c r="D31" s="30">
-        <f>IF(LEN(detail!R9)&lt;1,"",detail!R9)</f>
-        <v/>
-      </c>
-      <c r="E31" s="31" t="n"/>
+        <f>IF(LEN(detail!X8)&lt;1,"", detail!X8)</f>
+        <v/>
+      </c>
+      <c r="D31" s="31">
+        <f>IF(LEN(detail!R8)&lt;1,"",detail!R8)</f>
+        <v/>
+      </c>
+      <c r="E31" s="30" t="n"/>
       <c r="F31" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF9)&lt;1,"",detail!AF9), 0) &amp; IF(detail!AG9 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G31" s="30">
-        <f>IF(LEN(detail!AC9)&lt;1,"",detail!AC9)</f>
+        <f>DOLLAR(IF(LEN(detail!AF8)&lt;1,"",detail!AF8), 0) &amp; IF(detail!AG8 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G31" s="31">
+        <f>IF(LEN(detail!AC8)&lt;1,"",detail!AC8)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="14">
-        <f>IF(LEN(detail!P10)&lt;1,"",detail!P10)</f>
+        <f>IF(LEN(detail!P9)&lt;1,"",detail!P9)</f>
         <v/>
       </c>
       <c r="C32" s="14">
-        <f>IF(LEN(detail!X10)&lt;1,"", detail!X10)</f>
-        <v/>
-      </c>
-      <c r="D32" s="30">
-        <f>IF(LEN(detail!R10)&lt;1,"",detail!R10)</f>
-        <v/>
-      </c>
-      <c r="E32" s="31" t="n"/>
+        <f>IF(LEN(detail!X9)&lt;1,"", detail!X9)</f>
+        <v/>
+      </c>
+      <c r="D32" s="31">
+        <f>IF(LEN(detail!R9)&lt;1,"",detail!R9)</f>
+        <v/>
+      </c>
+      <c r="E32" s="30" t="n"/>
       <c r="F32" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF10)&lt;1,"",detail!AF10), 0) &amp; IF(detail!AG10 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G32" s="30">
-        <f>IF(LEN(detail!AC10)&lt;1,"",detail!AC10)</f>
+        <f>DOLLAR(IF(LEN(detail!AF9)&lt;1,"",detail!AF9), 0) &amp; IF(detail!AG9 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G32" s="31">
+        <f>IF(LEN(detail!AC9)&lt;1,"",detail!AC9)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="14">
-        <f>IF(LEN(detail!P11)&lt;1,"",detail!P11)</f>
+        <f>IF(LEN(detail!P10)&lt;1,"",detail!P10)</f>
         <v/>
       </c>
       <c r="C33" s="14">
-        <f>IF(LEN(detail!X11)&lt;1,"", detail!X11)</f>
-        <v/>
-      </c>
-      <c r="D33" s="30">
-        <f>IF(LEN(detail!R11)&lt;1,"",detail!R11)</f>
-        <v/>
-      </c>
-      <c r="E33" s="31" t="n"/>
+        <f>IF(LEN(detail!X10)&lt;1,"", detail!X10)</f>
+        <v/>
+      </c>
+      <c r="D33" s="31">
+        <f>IF(LEN(detail!R10)&lt;1,"",detail!R10)</f>
+        <v/>
+      </c>
+      <c r="E33" s="30" t="n"/>
       <c r="F33" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF11)&lt;1,"",detail!AF11), 0) &amp; IF(detail!AG11 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G33" s="30">
-        <f>IF(LEN(detail!AC11)&lt;1,"",detail!AC11)</f>
+        <f>DOLLAR(IF(LEN(detail!AF10)&lt;1,"",detail!AF10), 0) &amp; IF(detail!AG10 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G33" s="31">
+        <f>IF(LEN(detail!AC10)&lt;1,"",detail!AC10)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="14">
-        <f>IF(LEN(detail!P12)&lt;1,"",detail!P12)</f>
+        <f>IF(LEN(detail!P11)&lt;1,"",detail!P11)</f>
         <v/>
       </c>
       <c r="C34" s="14">
-        <f>IF(LEN(detail!X12)&lt;1,"", detail!X12)</f>
-        <v/>
-      </c>
-      <c r="D34" s="30">
-        <f>IF(LEN(detail!R12)&lt;1,"",detail!R12)</f>
-        <v/>
-      </c>
-      <c r="E34" s="31" t="n"/>
+        <f>IF(LEN(detail!X11)&lt;1,"", detail!X11)</f>
+        <v/>
+      </c>
+      <c r="D34" s="31">
+        <f>IF(LEN(detail!R11)&lt;1,"",detail!R11)</f>
+        <v/>
+      </c>
+      <c r="E34" s="30" t="n"/>
       <c r="F34" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF12)&lt;1,"",detail!AF12), 0) &amp; IF(detail!AG12 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G34" s="30">
-        <f>IF(LEN(detail!AC12)&lt;1,"",detail!AC12)</f>
+        <f>DOLLAR(IF(LEN(detail!AF11)&lt;1,"",detail!AF11), 0) &amp; IF(detail!AG11 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G34" s="31">
+        <f>IF(LEN(detail!AC11)&lt;1,"",detail!AC11)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="14">
-        <f>IF(LEN(detail!P13)&lt;1,"",detail!P13)</f>
+        <f>IF(LEN(detail!P12)&lt;1,"",detail!P12)</f>
         <v/>
       </c>
       <c r="C35" s="14">
-        <f>IF(LEN(detail!X13)&lt;1,"", detail!X13)</f>
-        <v/>
-      </c>
-      <c r="D35" s="30">
-        <f>IF(LEN(detail!R13)&lt;1,"",detail!R13)</f>
-        <v/>
-      </c>
-      <c r="E35" s="31" t="n"/>
+        <f>IF(LEN(detail!X12)&lt;1,"", detail!X12)</f>
+        <v/>
+      </c>
+      <c r="D35" s="31">
+        <f>IF(LEN(detail!R12)&lt;1,"",detail!R12)</f>
+        <v/>
+      </c>
+      <c r="E35" s="30" t="n"/>
       <c r="F35" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF13)&lt;1,"",detail!AF13), 0) &amp; IF(detail!AG13 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G35" s="30">
-        <f>IF(LEN(detail!AC13)&lt;1,"",detail!AC13)</f>
+        <f>DOLLAR(IF(LEN(detail!AF12)&lt;1,"",detail!AF12), 0) &amp; IF(detail!AG12 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G35" s="31">
+        <f>IF(LEN(detail!AC12)&lt;1,"",detail!AC12)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="14">
-        <f>IF(LEN(detail!P14)&lt;1,"",detail!P14)</f>
+        <f>IF(LEN(detail!P13)&lt;1,"",detail!P13)</f>
         <v/>
       </c>
       <c r="C36" s="14">
-        <f>IF(LEN(detail!X14)&lt;1,"", detail!X14)</f>
-        <v/>
-      </c>
-      <c r="D36" s="30">
-        <f>IF(LEN(detail!R14)&lt;1,"",detail!R14)</f>
-        <v/>
-      </c>
-      <c r="E36" s="31" t="n"/>
+        <f>IF(LEN(detail!X13)&lt;1,"", detail!X13)</f>
+        <v/>
+      </c>
+      <c r="D36" s="31">
+        <f>IF(LEN(detail!R13)&lt;1,"",detail!R13)</f>
+        <v/>
+      </c>
+      <c r="E36" s="30" t="n"/>
       <c r="F36" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF14)&lt;1,"",detail!AF14), 0) &amp; IF(detail!AG14 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G36" s="30">
-        <f>IF(LEN(detail!AC14)&lt;1,"",detail!AC14)</f>
+        <f>DOLLAR(IF(LEN(detail!AF13)&lt;1,"",detail!AF13), 0) &amp; IF(detail!AG13 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G36" s="31">
+        <f>IF(LEN(detail!AC13)&lt;1,"",detail!AC13)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="14">
-        <f>IF(LEN(detail!P15)&lt;1,"",detail!P15)</f>
+        <f>IF(LEN(detail!P14)&lt;1,"",detail!P14)</f>
         <v/>
       </c>
       <c r="C37" s="14">
-        <f>IF(LEN(detail!X15)&lt;1,"", detail!X15)</f>
-        <v/>
-      </c>
-      <c r="D37" s="30">
-        <f>IF(LEN(detail!R15)&lt;1,"",detail!R15)</f>
-        <v/>
-      </c>
-      <c r="E37" s="31" t="n"/>
+        <f>IF(LEN(detail!X14)&lt;1,"", detail!X14)</f>
+        <v/>
+      </c>
+      <c r="D37" s="31">
+        <f>IF(LEN(detail!R14)&lt;1,"",detail!R14)</f>
+        <v/>
+      </c>
+      <c r="E37" s="30" t="n"/>
       <c r="F37" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF15)&lt;1,"",detail!AF15), 0) &amp; IF(detail!AG15 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G37" s="30">
-        <f>IF(LEN(detail!AC15)&lt;1,"",detail!AC15)</f>
+        <f>DOLLAR(IF(LEN(detail!AF14)&lt;1,"",detail!AF14), 0) &amp; IF(detail!AG14 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G37" s="31">
+        <f>IF(LEN(detail!AC14)&lt;1,"",detail!AC14)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="14">
-        <f>IF(LEN(detail!P16)&lt;1,"",detail!P16)</f>
+        <f>IF(LEN(detail!P15)&lt;1,"",detail!P15)</f>
         <v/>
       </c>
       <c r="C38" s="14">
-        <f>IF(LEN(detail!X16)&lt;1,"", detail!X16)</f>
-        <v/>
-      </c>
-      <c r="D38" s="30">
-        <f>IF(LEN(detail!R16)&lt;1,"",detail!R16)</f>
-        <v/>
-      </c>
-      <c r="E38" s="31" t="n"/>
+        <f>IF(LEN(detail!X15)&lt;1,"", detail!X15)</f>
+        <v/>
+      </c>
+      <c r="D38" s="31">
+        <f>IF(LEN(detail!R15)&lt;1,"",detail!R15)</f>
+        <v/>
+      </c>
+      <c r="E38" s="30" t="n"/>
       <c r="F38" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF16)&lt;1,"",detail!AF16), 0) &amp; IF(detail!AG16 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G38" s="30">
-        <f>IF(LEN(detail!AC16)&lt;1,"",detail!AC16)</f>
+        <f>DOLLAR(IF(LEN(detail!AF15)&lt;1,"",detail!AF15), 0) &amp; IF(detail!AG15 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G38" s="31">
+        <f>IF(LEN(detail!AC15)&lt;1,"",detail!AC15)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="14">
-        <f>IF(LEN(detail!P17)&lt;1,"",detail!P17)</f>
+        <f>IF(LEN(detail!P16)&lt;1,"",detail!P16)</f>
         <v/>
       </c>
       <c r="C39" s="14">
-        <f>IF(LEN(detail!X17)&lt;1,"", detail!X17)</f>
-        <v/>
-      </c>
-      <c r="D39" s="30">
-        <f>IF(LEN(detail!R17)&lt;1,"",detail!R17)</f>
-        <v/>
-      </c>
-      <c r="E39" s="31" t="n"/>
+        <f>IF(LEN(detail!X16)&lt;1,"", detail!X16)</f>
+        <v/>
+      </c>
+      <c r="D39" s="31">
+        <f>IF(LEN(detail!R16)&lt;1,"",detail!R16)</f>
+        <v/>
+      </c>
+      <c r="E39" s="30" t="n"/>
       <c r="F39" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF17)&lt;1,"",detail!AF17), 0) &amp; IF(detail!AG17 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G39" s="30">
-        <f>IF(LEN(detail!AC17)&lt;1,"",detail!AC17)</f>
+        <f>DOLLAR(IF(LEN(detail!AF16)&lt;1,"",detail!AF16), 0) &amp; IF(detail!AG16 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G39" s="31">
+        <f>IF(LEN(detail!AC16)&lt;1,"",detail!AC16)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="14">
-        <f>IF(LEN(detail!P18)&lt;1,"",detail!P18)</f>
+        <f>IF(LEN(detail!P17)&lt;1,"",detail!P17)</f>
         <v/>
       </c>
       <c r="C40" s="14">
-        <f>IF(LEN(detail!X18)&lt;1,"", detail!X18)</f>
-        <v/>
-      </c>
-      <c r="D40" s="30">
-        <f>IF(LEN(detail!R18)&lt;1,"",detail!R18)</f>
-        <v/>
-      </c>
-      <c r="E40" s="31" t="n"/>
+        <f>IF(LEN(detail!X17)&lt;1,"", detail!X17)</f>
+        <v/>
+      </c>
+      <c r="D40" s="31">
+        <f>IF(LEN(detail!R17)&lt;1,"",detail!R17)</f>
+        <v/>
+      </c>
+      <c r="E40" s="30" t="n"/>
       <c r="F40" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF18)&lt;1,"",detail!AF18), 0) &amp; IF(detail!AG18 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G40" s="30">
-        <f>IF(LEN(detail!AC18)&lt;1,"",detail!AC18)</f>
+        <f>DOLLAR(IF(LEN(detail!AF17)&lt;1,"",detail!AF17), 0) &amp; IF(detail!AG17 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G40" s="31">
+        <f>IF(LEN(detail!AC17)&lt;1,"",detail!AC17)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="14">
-        <f>IF(LEN(detail!P19)&lt;1,"",detail!P19)</f>
+        <f>IF(LEN(detail!P18)&lt;1,"",detail!P18)</f>
         <v/>
       </c>
       <c r="C41" s="14">
-        <f>IF(LEN(detail!X19)&lt;1,"", detail!X19)</f>
-        <v/>
-      </c>
-      <c r="D41" s="30">
-        <f>IF(LEN(detail!R19)&lt;1,"",detail!R19)</f>
-        <v/>
-      </c>
-      <c r="E41" s="31" t="n"/>
+        <f>IF(LEN(detail!X18)&lt;1,"", detail!X18)</f>
+        <v/>
+      </c>
+      <c r="D41" s="31">
+        <f>IF(LEN(detail!R18)&lt;1,"",detail!R18)</f>
+        <v/>
+      </c>
+      <c r="E41" s="30" t="n"/>
       <c r="F41" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF19)&lt;1,"",detail!AF19), 0) &amp; IF(detail!AG19 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G41" s="30">
-        <f>IF(LEN(detail!AC19)&lt;1,"",detail!AC19)</f>
+        <f>DOLLAR(IF(LEN(detail!AF18)&lt;1,"",detail!AF18), 0) &amp; IF(detail!AG18 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G41" s="31">
+        <f>IF(LEN(detail!AC18)&lt;1,"",detail!AC18)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="14">
-        <f>IF(LEN(detail!P20)&lt;1,"",detail!P20)</f>
+        <f>IF(LEN(detail!P19)&lt;1,"",detail!P19)</f>
         <v/>
       </c>
       <c r="C42" s="14">
-        <f>IF(LEN(detail!X20)&lt;1,"", detail!X20)</f>
-        <v/>
-      </c>
-      <c r="D42" s="30">
-        <f>IF(LEN(detail!R20)&lt;1,"",detail!R20)</f>
-        <v/>
-      </c>
-      <c r="E42" s="31" t="n"/>
+        <f>IF(LEN(detail!X19)&lt;1,"", detail!X19)</f>
+        <v/>
+      </c>
+      <c r="D42" s="31">
+        <f>IF(LEN(detail!R19)&lt;1,"",detail!R19)</f>
+        <v/>
+      </c>
+      <c r="E42" s="30" t="n"/>
       <c r="F42" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF20)&lt;1,"",detail!AF20), 0) &amp; IF(detail!AG20 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G42" s="30">
-        <f>IF(LEN(detail!AC20)&lt;1,"",detail!AC20)</f>
+        <f>DOLLAR(IF(LEN(detail!AF19)&lt;1,"",detail!AF19), 0) &amp; IF(detail!AG19 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G42" s="31">
+        <f>IF(LEN(detail!AC19)&lt;1,"",detail!AC19)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="14">
-        <f>IF(LEN(detail!P21)&lt;1,"",detail!P21)</f>
+        <f>IF(LEN(detail!P20)&lt;1,"",detail!P20)</f>
         <v/>
       </c>
       <c r="C43" s="14">
-        <f>IF(LEN(detail!X21)&lt;1,"", detail!X21)</f>
-        <v/>
-      </c>
-      <c r="D43" s="30">
-        <f>IF(LEN(detail!R21)&lt;1,"",detail!R21)</f>
-        <v/>
-      </c>
-      <c r="E43" s="31" t="n"/>
+        <f>IF(LEN(detail!X20)&lt;1,"", detail!X20)</f>
+        <v/>
+      </c>
+      <c r="D43" s="31">
+        <f>IF(LEN(detail!R20)&lt;1,"",detail!R20)</f>
+        <v/>
+      </c>
+      <c r="E43" s="30" t="n"/>
       <c r="F43" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF21)&lt;1,"",detail!AF21), 0) &amp; IF(detail!AG21 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G43" s="30">
-        <f>IF(LEN(detail!AC21)&lt;1,"",detail!AC21)</f>
+        <f>DOLLAR(IF(LEN(detail!AF20)&lt;1,"",detail!AF20), 0) &amp; IF(detail!AG20 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G43" s="31">
+        <f>IF(LEN(detail!AC20)&lt;1,"",detail!AC20)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="14">
-        <f>IF(LEN(detail!P22)&lt;1,"",detail!P22)</f>
+        <f>IF(LEN(detail!P21)&lt;1,"",detail!P21)</f>
         <v/>
       </c>
       <c r="C44" s="14">
-        <f>IF(LEN(detail!X22)&lt;1,"", detail!X22)</f>
-        <v/>
-      </c>
-      <c r="D44" s="30">
-        <f>IF(LEN(detail!R22)&lt;1,"",detail!R22)</f>
-        <v/>
-      </c>
-      <c r="E44" s="31" t="n"/>
+        <f>IF(LEN(detail!X21)&lt;1,"", detail!X21)</f>
+        <v/>
+      </c>
+      <c r="D44" s="31">
+        <f>IF(LEN(detail!R21)&lt;1,"",detail!R21)</f>
+        <v/>
+      </c>
+      <c r="E44" s="30" t="n"/>
       <c r="F44" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF22)&lt;1,"",detail!AF22), 0) &amp; IF(detail!AG22 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G44" s="30">
-        <f>IF(LEN(detail!AC22)&lt;1,"",detail!AC22)</f>
+        <f>DOLLAR(IF(LEN(detail!AF21)&lt;1,"",detail!AF21), 0) &amp; IF(detail!AG21 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G44" s="31">
+        <f>IF(LEN(detail!AC21)&lt;1,"",detail!AC21)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="14">
+        <f>IF(LEN(detail!P22)&lt;1,"",detail!P22)</f>
+        <v/>
+      </c>
+      <c r="C45" s="14">
+        <f>IF(LEN(detail!X22)&lt;1,"", detail!X22)</f>
+        <v/>
+      </c>
+      <c r="D45" s="31">
+        <f>IF(LEN(detail!R22)&lt;1,"",detail!R22)</f>
+        <v/>
+      </c>
+      <c r="E45" s="30" t="n"/>
+      <c r="F45" s="9">
+        <f>DOLLAR(IF(LEN(detail!AF22)&lt;1,"",detail!AF22), 0) &amp; IF(detail!AG22 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G45" s="31">
+        <f>IF(LEN(detail!AC22)&lt;1,"",detail!AC22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="14">
         <f>IF(LEN(detail!P23)&lt;1,"",detail!P23)</f>
         <v/>
       </c>
-      <c r="C45" s="14">
+      <c r="C46" s="14">
         <f>IF(LEN(detail!X23)&lt;1,"", detail!X23)</f>
         <v/>
       </c>
-      <c r="D45" s="30">
+      <c r="D46" s="31">
         <f>IF(LEN(detail!R23)&lt;1,"",detail!R23)</f>
         <v/>
       </c>
-      <c r="E45" s="31" t="n"/>
-      <c r="F45" s="9">
+      <c r="E46" s="30" t="n"/>
+      <c r="F46" s="9">
         <f>DOLLAR(IF(LEN(detail!AF23)&lt;1,"",detail!AF23), 0) &amp; IF(detail!AG23 = 1, "*", "")</f>
         <v/>
       </c>
-      <c r="G45" s="30">
+      <c r="G46" s="31">
         <f>IF(LEN(detail!AC23)&lt;1,"",detail!AC23)</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="1" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="1" t="inlineStr">
         <is>
           <t>* An asterisk denotes that the opp includes a rebate</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="37">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B23:G23"/>
     <mergeCell ref="E9:G9"/>
+    <mergeCell ref="D46:E46"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="D36:E36"/>
+    <mergeCell ref="E17:F17"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="E17:F17"/>
     <mergeCell ref="D45:E45"/>
+    <mergeCell ref="E20:F20"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="E13:F13"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="D43:E43"/>
@@ -1871,23 +1954,20 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D30:E30"/>
     <mergeCell ref="D24:E24"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="B22:G22"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D38:E38"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D26:E26"/>
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D35:E35"/>
   </mergeCells>
-  <conditionalFormatting sqref="B24:D45 F24:G45">
+  <conditionalFormatting sqref="B25:D46 F25:G46">
     <cfRule type="containsErrors" priority="1" dxfId="0">
-      <formula>ISERROR(B24)</formula>
+      <formula>ISERROR(B25)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1902,7 +1982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1955,7 +2035,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1974,7 +2054,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>70000</v>
+        <v>123000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1990,7 +2070,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2009,11 +2089,11 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>70000</v>
+        <v>60000</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>L1_REV</t>
+          <t>ATM_ACCOUNT_REV</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2105,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2044,11 +2124,11 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>10500</v>
+        <v>9000</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>L1_PO</t>
+          <t>ATM_ACCOUNT_PO</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2140,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2079,11 +2159,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>63000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>L2_REV</t>
+          <t>L1_REV</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2175,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2114,11 +2194,11 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>9450</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>L2_PO</t>
+          <t>L1_PO</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2210,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2153,7 +2233,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CPAS_PO</t>
+          <t>L2_REV</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2245,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2188,7 +2268,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMPLANT_ACCEL_TRUE_UP</t>
+          <t>L2_PO</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2280,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2219,11 +2299,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PROGRAM_ACCEL_PO</t>
+          <t>CPAS_PO</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2315,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2254,11 +2334,11 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>10500</v>
+        <v>0</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>TTL_PO</t>
+          <t>IMPLANT_ACCEL_TRUE_UP</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2350,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2289,11 +2369,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>GUR_AMT</t>
+          <t>PROGRAM_ACCEL_PO</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2385,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2324,11 +2404,11 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>10500</v>
+        <v>18950</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PO_AMT</t>
+          <t>TTL_PO</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2420,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2359,11 +2439,11 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>IMPLANT_UNITS</t>
+          <t>GUR_AMT</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2455,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2394,11 +2474,11 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>18950</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>REVENUE_UNITS</t>
+          <t>PO_AMT</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2490,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2429,11 +2509,11 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>70000</v>
+        <v>4</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>QTD_SALES</t>
+          <t>IMPLANT_UNITS</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2525,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2464,11 +2544,11 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>QTD_IMPL_REV_RATIO</t>
+          <t>REVENUE_UNITS</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2560,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2499,9 +2579,79 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>10500</v>
+        <v>123000</v>
       </c>
       <c r="G17" t="inlineStr">
+        <is>
+          <t>QTD_SALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jmalberg@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026_Q1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>QTD_IMPL_REV_RATIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jmalberg@cvrx.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026_Q1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>18950</v>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>YTD_PO</t>
         </is>
@@ -2533,7 +2683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Y-Lan Cruea</t>
+          <t>Jennifer Malberg</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2695,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2569,7 +2719,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ORANGE COUNTY (CRUEA)</t>
+          <t>NORTH CALIFORNIA (MALBERG)</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2754,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>148500</v>
+        <v>170362.5</v>
       </c>
     </row>
     <row r="8">
@@ -2614,7 +2764,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>165000</v>
+        <v>245322</v>
       </c>
     </row>
     <row r="21" ht="15.95" customHeight="1"/>
@@ -2632,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AU4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2833,25 +2983,40 @@
       </c>
       <c r="AN1" t="inlineStr">
         <is>
+          <t>ATM_EMAIL</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>ATM_ACCOUNT_REVENUE</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
           <t>L1_REV</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>L2_REV</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>QTD_IMPL_REV_RATIO</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>ATM_ACCOUNT_PO</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
         <is>
           <t>L1_PO</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>L2_PO</t>
         </is>
@@ -2860,12 +3025,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Y-Lan Cruea</t>
+          <t>Jennifer Malberg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2875,17 +3040,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2898,8 +3063,8 @@
           <t>RE_07</t>
         </is>
       </c>
-      <c r="I2" s="48" t="n">
-        <v>46036</v>
+      <c r="I2" s="52" t="n">
+        <v>46048</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2923,32 +3088,32 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Providence Swedish (FKA Providence)</t>
+          <t>University of California Health (AKA UC Health-CA)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>St Joseph Hospital Orange</t>
+          <t>Ucsf Medical Center</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>0014u00001pyTy3AAE</t>
+          <t>0014u00001pyZlqAAE</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>CRX773 029408</t>
+          <t>CVR314 028890</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>006UY00000VM5GwYAL</t>
+          <t>006UY00000U3JknYAF</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -2982,57 +3147,63 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AF2" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH2" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AI2" t="n">
-        <v>148500</v>
+        <v>170362.5</v>
       </c>
       <c r="AJ2" t="n">
-        <v>165000</v>
+        <v>245322</v>
       </c>
       <c r="AK2" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AL2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM2" t="n">
         <v>1</v>
       </c>
-      <c r="AN2" t="n">
-        <v>35000</v>
-      </c>
       <c r="AO2" t="n">
         <v>0</v>
       </c>
       <c r="AP2" t="n">
+        <v>31500</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>0</v>
       </c>
-      <c r="AQ2" t="n">
-        <v>5250</v>
-      </c>
       <c r="AR2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>4725</v>
+      </c>
+      <c r="AU2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Y-Lan Cruea</t>
+          <t>Jennifer Malberg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3042,17 +3213,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TERR_26</t>
+          <t>TERR_37</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3065,8 +3236,8 @@
           <t>RE_07</t>
         </is>
       </c>
-      <c r="I3" s="48" t="n">
-        <v>46052</v>
+      <c r="I3" s="52" t="n">
+        <v>46048</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -3090,32 +3261,32 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Providence Swedish (FKA Providence)</t>
+          <t>University of California Health (AKA UC Health-CA)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>St Joseph Hospital Orange</t>
+          <t>Ucsf Medical Center</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>0014u00001pyTy3AAE</t>
+          <t>0014u00001pyZlqAAE</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>CRX773 029676</t>
+          <t>CVR314 029551</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>006UY00000VvRzKYAV</t>
+          <t>006UY00000VfcIoYAJ</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ycruea@cvrx.com</t>
+          <t>jmalberg@cvrx.com</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -3149,45 +3320,229 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AF3" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH3" t="n">
-        <v>35000</v>
+        <v>31500</v>
       </c>
       <c r="AI3" t="n">
-        <v>148500</v>
+        <v>170362.5</v>
       </c>
       <c r="AJ3" t="n">
-        <v>165000</v>
+        <v>245322</v>
       </c>
       <c r="AK3" t="n">
-        <v>70000</v>
+        <v>63000</v>
       </c>
       <c r="AL3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM3" t="n">
         <v>2</v>
       </c>
-      <c r="AN3" t="n">
-        <v>35000</v>
-      </c>
       <c r="AO3" t="n">
         <v>0</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.5</v>
+        <v>31500</v>
       </c>
       <c r="AQ3" t="n">
-        <v>5250</v>
+        <v>0</v>
       </c>
       <c r="AR3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>4725</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jmalberg@cvrx.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jennifer Malberg</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TERR_37</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TERR_37</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TERR_37</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PACIFIC</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>RE_07</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="n">
+        <v>46053</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026_01</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026_Q1</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026_02</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026_Q1</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Kaweah Health (FKA Kaweah Delta Health Care District)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Kaweah Delta Medical Center</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0014u00001s9EpwAAE</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>CRX305 029860</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>006UY00000WRIhZYAX</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>jmalberg@cvrx.com</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Heart Failure - Reduced Ejection Fraction</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>De novo</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Revenue Recognized</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>170362.5</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>245322</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>123000</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>brummonds@cvrx.com</t>
+        </is>
+      </c>
+      <c r="AO4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>9000</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
simplify and add recoverable draw to TM statements
</commit_message>
<xml_diff>
--- a/Excel Files/COMP_STATEMENT.xlsx
+++ b/Excel Files/COMP_STATEMENT.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +89,15 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -122,7 +131,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -483,14 +492,27 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="hair">
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="hair">
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -527,6 +549,17 @@
     <border>
       <left/>
       <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
         <color indexed="64"/>
       </right>
       <top style="medium">
@@ -570,7 +603,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -638,15 +671,31 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -661,29 +710,31 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1084,16 +1135,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K47"/>
+  <dimension ref="A2:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
-    <col width="0.7109375" customWidth="1" style="1" min="1" max="1"/>
-    <col width="25.28515625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="13.7109375" customWidth="1" style="1" min="3" max="3"/>
-    <col width="11.85546875" customWidth="1" style="1" min="4" max="4"/>
-    <col width="5.5703125" customWidth="1" style="1" min="5" max="5"/>
-    <col width="17.85546875" customWidth="1" style="1" min="6" max="6"/>
-    <col width="14.7109375" customWidth="1" style="1" min="7" max="7"/>
+    <col width="0.7109375" customWidth="1" style="39" min="1" max="1"/>
+    <col width="25.28515625" customWidth="1" style="39" min="2" max="2"/>
+    <col width="13.7109375" customWidth="1" style="39" min="3" max="3"/>
+    <col width="11.85546875" customWidth="1" style="39" min="4" max="4"/>
+    <col width="5.5703125" customWidth="1" style="39" min="5" max="5"/>
+    <col width="17.85546875" customWidth="1" style="39" min="6" max="6"/>
+    <col width="14.7109375" customWidth="1" style="39" min="7" max="7"/>
     <col width="12.5703125" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -1131,28 +1182,28 @@
     <row r="7" ht="3.95" customHeight="1"/>
     <row r="8" ht="3.95" customHeight="1" thickBot="1"/>
     <row r="9">
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="40" t="inlineStr">
         <is>
           <t>Sales Performance</t>
         </is>
       </c>
-      <c r="C9" s="36" t="n"/>
+      <c r="C9" s="42" t="n"/>
       <c r="D9" s="3" t="n"/>
-      <c r="E9" s="34" t="inlineStr">
+      <c r="E9" s="40" t="inlineStr">
         <is>
           <t>Final Payment</t>
         </is>
       </c>
-      <c r="F9" s="35" t="n"/>
-      <c r="G9" s="36" t="n"/>
+      <c r="F9" s="41" t="n"/>
+      <c r="G9" s="42" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>ATM Account Sales</t>
         </is>
       </c>
-      <c r="C10" s="50">
+      <c r="C10" s="30">
         <f>_xlfn.XLOOKUP("ATM_ACCOUNT_REV", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
@@ -1160,13 +1211,13 @@
         <f>IF(G10&gt;0, 1, 0)</f>
         <v/>
       </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="E10" s="48" t="inlineStr">
         <is>
           <t>ATM Account Payout</t>
         </is>
       </c>
-      <c r="F10" s="30" t="n"/>
-      <c r="G10" s="49">
+      <c r="F10" s="36" t="n"/>
+      <c r="G10" s="29">
         <f>_xlfn.XLOOKUP("ATM_ACCOUNT_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
@@ -1176,7 +1227,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Level 1 Sales</t>
         </is>
@@ -1186,12 +1237,12 @@
         <v/>
       </c>
       <c r="D11" s="5" t="n"/>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="E11" s="35" t="inlineStr">
         <is>
           <t>Level 1 Payout</t>
         </is>
       </c>
-      <c r="F11" s="30" t="n"/>
+      <c r="F11" s="36" t="n"/>
       <c r="G11" s="6">
         <f>_xlfn.XLOOKUP("L1_PO", payout!G:G,payout!F:F)</f>
         <v/>
@@ -1203,7 +1254,7 @@
     </row>
     <row r="12" ht="16.5" customHeight="1" thickBot="1">
       <c r="A12" s="5" t="n"/>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Level 2 Sales</t>
         </is>
@@ -1213,12 +1264,12 @@
         <v/>
       </c>
       <c r="D12" s="5" t="n"/>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>Level 2 Payout</t>
         </is>
       </c>
-      <c r="F12" s="30" t="n"/>
+      <c r="F12" s="36" t="n"/>
       <c r="G12" s="12">
         <f>_xlfn.XLOOKUP("L2_PO",payout!G:G,payout!F:F)</f>
         <v/>
@@ -1239,12 +1290,12 @@
         <v/>
       </c>
       <c r="D13" s="5" t="n"/>
-      <c r="E13" s="43" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="F13" s="44" t="n"/>
+      <c r="F13" s="50" t="n"/>
       <c r="G13" s="13">
         <f>SUM(G10:G12)</f>
         <v/>
@@ -1262,12 +1313,12 @@
         <v/>
       </c>
       <c r="D14" s="5" t="n"/>
-      <c r="E14" s="37" t="inlineStr">
+      <c r="E14" s="43" t="inlineStr">
         <is>
           <t>Adjustments</t>
         </is>
       </c>
-      <c r="F14" s="38" t="n"/>
+      <c r="F14" s="44" t="n"/>
       <c r="G14" s="11">
         <f>_xlfn.IFNA(_xlfn.XLOOKUP("ADJUSTMENTS", payout!G:G,payout!F:F), 0) + _xlfn.IFNA(_xlfn.XLOOKUP("T-SPLIT", payout!G:G,payout!F:F), 0)</f>
         <v/>
@@ -1277,12 +1328,12 @@
       <c r="D15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="45" t="inlineStr">
+      <c r="E15" s="53" t="inlineStr">
         <is>
           <t>CPAS Payout</t>
         </is>
       </c>
-      <c r="F15" s="30" t="n"/>
+      <c r="F15" s="36" t="n"/>
       <c r="G15" s="11">
         <f>IFERROR(_xlfn.XLOOKUP("CPAS_PO", payout!G:G,payout!F:F), 0)</f>
         <v/>
@@ -1293,12 +1344,12 @@
         <f>IF(G16&gt;0, 1, 0)</f>
         <v/>
       </c>
-      <c r="E16" s="39" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>Program Accel</t>
         </is>
       </c>
-      <c r="F16" s="30" t="n"/>
+      <c r="F16" s="36" t="n"/>
       <c r="G16" s="11">
         <f>IFERROR(_xlfn.XLOOKUP("PROGRAM_ACCEL_PO",payout!G:G,payout!F:F), 0)</f>
         <v/>
@@ -1309,12 +1360,12 @@
         <f>IF(G17&gt;0, 1, 0)</f>
         <v/>
       </c>
-      <c r="E17" s="39" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>Implant Ratio Accel</t>
         </is>
       </c>
-      <c r="F17" s="30" t="n"/>
+      <c r="F17" s="36" t="n"/>
       <c r="G17" s="11">
         <f>IFERROR(_xlfn.XLOOKUP("IMPLANT_ACCEL_TRUE_UP",payout!G:G,payout!F:F), 0)</f>
         <v/>
@@ -1325,12 +1376,12 @@
         <f>IF(G18&gt;0, IF(G18&gt;IFERROR(_xlfn.XLOOKUP("TTL_PO", payout!G:G,payout!F:F), 0), 1, 0), 0)</f>
         <v/>
       </c>
-      <c r="E18" s="47" t="inlineStr">
+      <c r="E18" s="57" t="inlineStr">
         <is>
           <t>Minimum Payout</t>
         </is>
       </c>
-      <c r="F18" s="48" t="n"/>
+      <c r="F18" s="58" t="n"/>
       <c r="G18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP("GUR_AMT",payout!G:G,payout!F:F), 0)</f>
         <v/>
@@ -1338,12 +1389,12 @@
     </row>
     <row r="19" ht="17.25" customHeight="1" thickBot="1" thickTop="1">
       <c r="D19" s="24" t="n"/>
-      <c r="E19" s="43" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr">
         <is>
           <t>Final Payout</t>
         </is>
       </c>
-      <c r="F19" s="44" t="n"/>
+      <c r="F19" s="50" t="n"/>
       <c r="G19" s="26">
         <f>_xlfn.XLOOKUP("PO_AMT", payout!G:G,payout!F:F)</f>
         <v/>
@@ -1359,567 +1410,542 @@
         <f>info!B7</f>
         <v/>
       </c>
-      <c r="E20" s="40" t="inlineStr">
+      <c r="E20" s="46" t="inlineStr">
         <is>
           <t>YTD Payout</t>
         </is>
       </c>
-      <c r="F20" s="41" t="n"/>
+      <c r="F20" s="47" t="n"/>
       <c r="G20" s="17">
         <f>_xlfn.XLOOKUP("YTD_PO", payout!G:G,payout!F:F)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="3.95" customHeight="1"/>
-    <row r="22" ht="3.95" customHeight="1"/>
-    <row r="23">
-      <c r="B23" s="32" t="inlineStr">
+    <row r="21" ht="16.5" customHeight="1" thickBot="1">
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="G21" s="33" t="n"/>
+    </row>
+    <row r="22" ht="32.25" customHeight="1" thickBot="1">
+      <c r="B22" s="38" t="n"/>
+      <c r="D22" s="5">
+        <f>IF(G22&lt;&gt;0, 1, 0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="55" t="inlineStr">
+        <is>
+          <t>Recoverable Draw (estimated)</t>
+        </is>
+      </c>
+      <c r="F22" s="56" t="n"/>
+      <c r="G22" s="34">
+        <f>IFERROR(-info!B9, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Opportunity Detail </t>
         </is>
       </c>
-      <c r="C23" s="33" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
-      <c r="G23" s="30" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="46" t="inlineStr">
+      <c r="C24" s="52" t="n"/>
+      <c r="D24" s="52" t="n"/>
+      <c r="E24" s="52" t="n"/>
+      <c r="F24" s="52" t="n"/>
+      <c r="G24" s="36" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="54" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C24" s="46" t="inlineStr">
+      <c r="C25" s="54" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D24" s="46" t="inlineStr">
+      <c r="D25" s="54" t="inlineStr">
         <is>
           <t>Opp Name</t>
         </is>
       </c>
-      <c r="E24" s="30" t="n"/>
-      <c r="F24" s="46" t="inlineStr">
+      <c r="E25" s="36" t="n"/>
+      <c r="F25" s="54" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="G24" s="46" t="inlineStr">
+      <c r="G25" s="54" t="inlineStr">
         <is>
           <t>Rev Units</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="14">
-        <f>IF(LEN(detail!P2)&lt;1,"",detail!P2)</f>
-        <v/>
-      </c>
-      <c r="C25" s="14">
-        <f>IF(LEN(detail!X2)&lt;1,"", detail!X2)</f>
-        <v/>
-      </c>
-      <c r="D25" s="31">
-        <f>IF(LEN(detail!R2)&lt;1,"",detail!R2)</f>
-        <v/>
-      </c>
-      <c r="E25" s="30" t="n"/>
-      <c r="F25" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF2)&lt;1,"",detail!AF2), 0) &amp; IF(detail!AG2 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G25" s="31">
-        <f>IF(LEN(detail!AC2)&lt;1,"",detail!AC2)</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="14">
-        <f>IF(LEN(detail!P3)&lt;1,"",detail!P3)</f>
+        <f>IF(LEN(detail!P2)&lt;1,"",detail!P2)</f>
         <v/>
       </c>
       <c r="C26" s="14">
-        <f>IF(LEN(detail!X3)&lt;1,"", detail!X3)</f>
-        <v/>
-      </c>
-      <c r="D26" s="31">
-        <f>IF(LEN(detail!R3)&lt;1,"",detail!R3)</f>
-        <v/>
-      </c>
-      <c r="E26" s="30" t="n"/>
+        <f>IF(LEN(detail!X2)&lt;1,"", detail!X2)</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>IF(LEN(detail!R2)&lt;1,"",detail!R2)</f>
+        <v/>
+      </c>
+      <c r="E26" s="36" t="n"/>
       <c r="F26" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF3)&lt;1,"",detail!AF3), 0) &amp; IF(detail!AG3 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G26" s="31">
-        <f>IF(LEN(detail!AC3)&lt;1,"",detail!AC3)</f>
+        <f>DOLLAR(IF(LEN(detail!AF2)&lt;1,"",detail!AF2), 0) &amp; IF(detail!AG2 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G26" s="37">
+        <f>IF(LEN(detail!AC2)&lt;1,"",detail!AC2)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="14">
-        <f>IF(LEN(detail!P4)&lt;1,"",detail!P4)</f>
+        <f>IF(LEN(detail!P3)&lt;1,"",detail!P3)</f>
         <v/>
       </c>
       <c r="C27" s="14">
-        <f>IF(LEN(detail!X4)&lt;1,"", detail!X4)</f>
-        <v/>
-      </c>
-      <c r="D27" s="31">
-        <f>IF(LEN(detail!R4)&lt;1,"",detail!R4)</f>
-        <v/>
-      </c>
-      <c r="E27" s="30" t="n"/>
+        <f>IF(LEN(detail!X3)&lt;1,"", detail!X3)</f>
+        <v/>
+      </c>
+      <c r="D27" s="37">
+        <f>IF(LEN(detail!R3)&lt;1,"",detail!R3)</f>
+        <v/>
+      </c>
+      <c r="E27" s="36" t="n"/>
       <c r="F27" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF4)&lt;1,"",detail!AF4), 0) &amp; IF(detail!AG4 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G27" s="31">
-        <f>IF(LEN(detail!AC4)&lt;1,"",detail!AC4)</f>
+        <f>DOLLAR(IF(LEN(detail!AF3)&lt;1,"",detail!AF3), 0) &amp; IF(detail!AG3 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G27" s="37">
+        <f>IF(LEN(detail!AC3)&lt;1,"",detail!AC3)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="14">
-        <f>IF(LEN(detail!P5)&lt;1,"",detail!P5)</f>
+        <f>IF(LEN(detail!P4)&lt;1,"",detail!P4)</f>
         <v/>
       </c>
       <c r="C28" s="14">
-        <f>IF(LEN(detail!X5)&lt;1,"", detail!X5)</f>
-        <v/>
-      </c>
-      <c r="D28" s="31">
-        <f>IF(LEN(detail!R5)&lt;1,"",detail!R5)</f>
-        <v/>
-      </c>
-      <c r="E28" s="30" t="n"/>
+        <f>IF(LEN(detail!X4)&lt;1,"", detail!X4)</f>
+        <v/>
+      </c>
+      <c r="D28" s="37">
+        <f>IF(LEN(detail!R4)&lt;1,"",detail!R4)</f>
+        <v/>
+      </c>
+      <c r="E28" s="36" t="n"/>
       <c r="F28" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF5)&lt;1,"",detail!AF5), 0) &amp; IF(detail!AG5 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G28" s="31">
-        <f>IF(LEN(detail!AC5)&lt;1,"",detail!AC5)</f>
+        <f>DOLLAR(IF(LEN(detail!AF4)&lt;1,"",detail!AF4), 0) &amp; IF(detail!AG4 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G28" s="37">
+        <f>IF(LEN(detail!AC4)&lt;1,"",detail!AC4)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="14">
-        <f>IF(LEN(detail!P6)&lt;1,"",detail!P6)</f>
+        <f>IF(LEN(detail!P5)&lt;1,"",detail!P5)</f>
         <v/>
       </c>
       <c r="C29" s="14">
-        <f>IF(LEN(detail!X6)&lt;1,"", detail!X6)</f>
-        <v/>
-      </c>
-      <c r="D29" s="31">
-        <f>IF(LEN(detail!R6)&lt;1,"",detail!R6)</f>
-        <v/>
-      </c>
-      <c r="E29" s="30" t="n"/>
+        <f>IF(LEN(detail!X5)&lt;1,"", detail!X5)</f>
+        <v/>
+      </c>
+      <c r="D29" s="37">
+        <f>IF(LEN(detail!R5)&lt;1,"",detail!R5)</f>
+        <v/>
+      </c>
+      <c r="E29" s="36" t="n"/>
       <c r="F29" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF6)&lt;1,"",detail!AF6), 0) &amp; IF(detail!AG6 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G29" s="31">
-        <f>IF(LEN(detail!AC6)&lt;1,"",detail!AC6)</f>
+        <f>DOLLAR(IF(LEN(detail!AF5)&lt;1,"",detail!AF5), 0) &amp; IF(detail!AG5 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G29" s="37">
+        <f>IF(LEN(detail!AC5)&lt;1,"",detail!AC5)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="14">
-        <f>IF(LEN(detail!P7)&lt;1,"",detail!P7)</f>
+        <f>IF(LEN(detail!P6)&lt;1,"",detail!P6)</f>
         <v/>
       </c>
       <c r="C30" s="14">
-        <f>IF(LEN(detail!X7)&lt;1,"", detail!X7)</f>
-        <v/>
-      </c>
-      <c r="D30" s="31">
-        <f>IF(LEN(detail!R7)&lt;1,"",detail!R7)</f>
-        <v/>
-      </c>
-      <c r="E30" s="30" t="n"/>
+        <f>IF(LEN(detail!X6)&lt;1,"", detail!X6)</f>
+        <v/>
+      </c>
+      <c r="D30" s="37">
+        <f>IF(LEN(detail!R6)&lt;1,"",detail!R6)</f>
+        <v/>
+      </c>
+      <c r="E30" s="36" t="n"/>
       <c r="F30" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF7)&lt;1,"",detail!AF7), 0) &amp; IF(detail!AG7 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G30" s="31">
-        <f>IF(LEN(detail!AC7)&lt;1,"",detail!AC7)</f>
+        <f>DOLLAR(IF(LEN(detail!AF6)&lt;1,"",detail!AF6), 0) &amp; IF(detail!AG6 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G30" s="37">
+        <f>IF(LEN(detail!AC6)&lt;1,"",detail!AC6)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="14">
-        <f>IF(LEN(detail!P8)&lt;1,"",detail!P8)</f>
+        <f>IF(LEN(detail!P7)&lt;1,"",detail!P7)</f>
         <v/>
       </c>
       <c r="C31" s="14">
-        <f>IF(LEN(detail!X8)&lt;1,"", detail!X8)</f>
-        <v/>
-      </c>
-      <c r="D31" s="31">
-        <f>IF(LEN(detail!R8)&lt;1,"",detail!R8)</f>
-        <v/>
-      </c>
-      <c r="E31" s="30" t="n"/>
+        <f>IF(LEN(detail!X7)&lt;1,"", detail!X7)</f>
+        <v/>
+      </c>
+      <c r="D31" s="37">
+        <f>IF(LEN(detail!R7)&lt;1,"",detail!R7)</f>
+        <v/>
+      </c>
+      <c r="E31" s="36" t="n"/>
       <c r="F31" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF8)&lt;1,"",detail!AF8), 0) &amp; IF(detail!AG8 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G31" s="31">
-        <f>IF(LEN(detail!AC8)&lt;1,"",detail!AC8)</f>
+        <f>DOLLAR(IF(LEN(detail!AF7)&lt;1,"",detail!AF7), 0) &amp; IF(detail!AG7 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G31" s="37">
+        <f>IF(LEN(detail!AC7)&lt;1,"",detail!AC7)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="14">
-        <f>IF(LEN(detail!P9)&lt;1,"",detail!P9)</f>
+        <f>IF(LEN(detail!P8)&lt;1,"",detail!P8)</f>
         <v/>
       </c>
       <c r="C32" s="14">
-        <f>IF(LEN(detail!X9)&lt;1,"", detail!X9)</f>
-        <v/>
-      </c>
-      <c r="D32" s="31">
-        <f>IF(LEN(detail!R9)&lt;1,"",detail!R9)</f>
-        <v/>
-      </c>
-      <c r="E32" s="30" t="n"/>
+        <f>IF(LEN(detail!X8)&lt;1,"", detail!X8)</f>
+        <v/>
+      </c>
+      <c r="D32" s="37">
+        <f>IF(LEN(detail!R8)&lt;1,"",detail!R8)</f>
+        <v/>
+      </c>
+      <c r="E32" s="36" t="n"/>
       <c r="F32" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF9)&lt;1,"",detail!AF9), 0) &amp; IF(detail!AG9 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G32" s="31">
-        <f>IF(LEN(detail!AC9)&lt;1,"",detail!AC9)</f>
+        <f>DOLLAR(IF(LEN(detail!AF8)&lt;1,"",detail!AF8), 0) &amp; IF(detail!AG8 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G32" s="37">
+        <f>IF(LEN(detail!AC8)&lt;1,"",detail!AC8)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="14">
-        <f>IF(LEN(detail!P10)&lt;1,"",detail!P10)</f>
+        <f>IF(LEN(detail!P9)&lt;1,"",detail!P9)</f>
         <v/>
       </c>
       <c r="C33" s="14">
-        <f>IF(LEN(detail!X10)&lt;1,"", detail!X10)</f>
-        <v/>
-      </c>
-      <c r="D33" s="31">
-        <f>IF(LEN(detail!R10)&lt;1,"",detail!R10)</f>
-        <v/>
-      </c>
-      <c r="E33" s="30" t="n"/>
+        <f>IF(LEN(detail!X9)&lt;1,"", detail!X9)</f>
+        <v/>
+      </c>
+      <c r="D33" s="37">
+        <f>IF(LEN(detail!R9)&lt;1,"",detail!R9)</f>
+        <v/>
+      </c>
+      <c r="E33" s="36" t="n"/>
       <c r="F33" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF10)&lt;1,"",detail!AF10), 0) &amp; IF(detail!AG10 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G33" s="31">
-        <f>IF(LEN(detail!AC10)&lt;1,"",detail!AC10)</f>
+        <f>DOLLAR(IF(LEN(detail!AF9)&lt;1,"",detail!AF9), 0) &amp; IF(detail!AG9 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G33" s="37">
+        <f>IF(LEN(detail!AC9)&lt;1,"",detail!AC9)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="14">
-        <f>IF(LEN(detail!P11)&lt;1,"",detail!P11)</f>
+        <f>IF(LEN(detail!P10)&lt;1,"",detail!P10)</f>
         <v/>
       </c>
       <c r="C34" s="14">
-        <f>IF(LEN(detail!X11)&lt;1,"", detail!X11)</f>
-        <v/>
-      </c>
-      <c r="D34" s="31">
-        <f>IF(LEN(detail!R11)&lt;1,"",detail!R11)</f>
-        <v/>
-      </c>
-      <c r="E34" s="30" t="n"/>
+        <f>IF(LEN(detail!X10)&lt;1,"", detail!X10)</f>
+        <v/>
+      </c>
+      <c r="D34" s="37">
+        <f>IF(LEN(detail!R10)&lt;1,"",detail!R10)</f>
+        <v/>
+      </c>
+      <c r="E34" s="36" t="n"/>
       <c r="F34" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF11)&lt;1,"",detail!AF11), 0) &amp; IF(detail!AG11 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G34" s="31">
-        <f>IF(LEN(detail!AC11)&lt;1,"",detail!AC11)</f>
+        <f>DOLLAR(IF(LEN(detail!AF10)&lt;1,"",detail!AF10), 0) &amp; IF(detail!AG10 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G34" s="37">
+        <f>IF(LEN(detail!AC10)&lt;1,"",detail!AC10)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="14">
-        <f>IF(LEN(detail!P12)&lt;1,"",detail!P12)</f>
+        <f>IF(LEN(detail!P11)&lt;1,"",detail!P11)</f>
         <v/>
       </c>
       <c r="C35" s="14">
-        <f>IF(LEN(detail!X12)&lt;1,"", detail!X12)</f>
-        <v/>
-      </c>
-      <c r="D35" s="31">
-        <f>IF(LEN(detail!R12)&lt;1,"",detail!R12)</f>
-        <v/>
-      </c>
-      <c r="E35" s="30" t="n"/>
+        <f>IF(LEN(detail!X11)&lt;1,"", detail!X11)</f>
+        <v/>
+      </c>
+      <c r="D35" s="37">
+        <f>IF(LEN(detail!R11)&lt;1,"",detail!R11)</f>
+        <v/>
+      </c>
+      <c r="E35" s="36" t="n"/>
       <c r="F35" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF12)&lt;1,"",detail!AF12), 0) &amp; IF(detail!AG12 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G35" s="31">
-        <f>IF(LEN(detail!AC12)&lt;1,"",detail!AC12)</f>
+        <f>DOLLAR(IF(LEN(detail!AF11)&lt;1,"",detail!AF11), 0) &amp; IF(detail!AG11 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G35" s="37">
+        <f>IF(LEN(detail!AC11)&lt;1,"",detail!AC11)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="14">
-        <f>IF(LEN(detail!P13)&lt;1,"",detail!P13)</f>
+        <f>IF(LEN(detail!P12)&lt;1,"",detail!P12)</f>
         <v/>
       </c>
       <c r="C36" s="14">
-        <f>IF(LEN(detail!X13)&lt;1,"", detail!X13)</f>
-        <v/>
-      </c>
-      <c r="D36" s="31">
-        <f>IF(LEN(detail!R13)&lt;1,"",detail!R13)</f>
-        <v/>
-      </c>
-      <c r="E36" s="30" t="n"/>
+        <f>IF(LEN(detail!X12)&lt;1,"", detail!X12)</f>
+        <v/>
+      </c>
+      <c r="D36" s="37">
+        <f>IF(LEN(detail!R12)&lt;1,"",detail!R12)</f>
+        <v/>
+      </c>
+      <c r="E36" s="36" t="n"/>
       <c r="F36" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF13)&lt;1,"",detail!AF13), 0) &amp; IF(detail!AG13 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G36" s="31">
-        <f>IF(LEN(detail!AC13)&lt;1,"",detail!AC13)</f>
+        <f>DOLLAR(IF(LEN(detail!AF12)&lt;1,"",detail!AF12), 0) &amp; IF(detail!AG12 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G36" s="37">
+        <f>IF(LEN(detail!AC12)&lt;1,"",detail!AC12)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="14">
-        <f>IF(LEN(detail!P14)&lt;1,"",detail!P14)</f>
+        <f>IF(LEN(detail!P13)&lt;1,"",detail!P13)</f>
         <v/>
       </c>
       <c r="C37" s="14">
-        <f>IF(LEN(detail!X14)&lt;1,"", detail!X14)</f>
-        <v/>
-      </c>
-      <c r="D37" s="31">
-        <f>IF(LEN(detail!R14)&lt;1,"",detail!R14)</f>
-        <v/>
-      </c>
-      <c r="E37" s="30" t="n"/>
+        <f>IF(LEN(detail!X13)&lt;1,"", detail!X13)</f>
+        <v/>
+      </c>
+      <c r="D37" s="37">
+        <f>IF(LEN(detail!R13)&lt;1,"",detail!R13)</f>
+        <v/>
+      </c>
+      <c r="E37" s="36" t="n"/>
       <c r="F37" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF14)&lt;1,"",detail!AF14), 0) &amp; IF(detail!AG14 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G37" s="31">
-        <f>IF(LEN(detail!AC14)&lt;1,"",detail!AC14)</f>
+        <f>DOLLAR(IF(LEN(detail!AF13)&lt;1,"",detail!AF13), 0) &amp; IF(detail!AG13 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G37" s="37">
+        <f>IF(LEN(detail!AC13)&lt;1,"",detail!AC13)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="14">
-        <f>IF(LEN(detail!P15)&lt;1,"",detail!P15)</f>
+        <f>IF(LEN(detail!P14)&lt;1,"",detail!P14)</f>
         <v/>
       </c>
       <c r="C38" s="14">
-        <f>IF(LEN(detail!X15)&lt;1,"", detail!X15)</f>
-        <v/>
-      </c>
-      <c r="D38" s="31">
-        <f>IF(LEN(detail!R15)&lt;1,"",detail!R15)</f>
-        <v/>
-      </c>
-      <c r="E38" s="30" t="n"/>
+        <f>IF(LEN(detail!X14)&lt;1,"", detail!X14)</f>
+        <v/>
+      </c>
+      <c r="D38" s="37">
+        <f>IF(LEN(detail!R14)&lt;1,"",detail!R14)</f>
+        <v/>
+      </c>
+      <c r="E38" s="36" t="n"/>
       <c r="F38" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF15)&lt;1,"",detail!AF15), 0) &amp; IF(detail!AG15 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G38" s="31">
-        <f>IF(LEN(detail!AC15)&lt;1,"",detail!AC15)</f>
+        <f>DOLLAR(IF(LEN(detail!AF14)&lt;1,"",detail!AF14), 0) &amp; IF(detail!AG14 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G38" s="37">
+        <f>IF(LEN(detail!AC14)&lt;1,"",detail!AC14)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="14">
-        <f>IF(LEN(detail!P16)&lt;1,"",detail!P16)</f>
+        <f>IF(LEN(detail!P15)&lt;1,"",detail!P15)</f>
         <v/>
       </c>
       <c r="C39" s="14">
-        <f>IF(LEN(detail!X16)&lt;1,"", detail!X16)</f>
-        <v/>
-      </c>
-      <c r="D39" s="31">
-        <f>IF(LEN(detail!R16)&lt;1,"",detail!R16)</f>
-        <v/>
-      </c>
-      <c r="E39" s="30" t="n"/>
+        <f>IF(LEN(detail!X15)&lt;1,"", detail!X15)</f>
+        <v/>
+      </c>
+      <c r="D39" s="37">
+        <f>IF(LEN(detail!R15)&lt;1,"",detail!R15)</f>
+        <v/>
+      </c>
+      <c r="E39" s="36" t="n"/>
       <c r="F39" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF16)&lt;1,"",detail!AF16), 0) &amp; IF(detail!AG16 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G39" s="31">
-        <f>IF(LEN(detail!AC16)&lt;1,"",detail!AC16)</f>
+        <f>DOLLAR(IF(LEN(detail!AF15)&lt;1,"",detail!AF15), 0) &amp; IF(detail!AG15 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G39" s="37">
+        <f>IF(LEN(detail!AC15)&lt;1,"",detail!AC15)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="14">
-        <f>IF(LEN(detail!P17)&lt;1,"",detail!P17)</f>
+        <f>IF(LEN(detail!P16)&lt;1,"",detail!P16)</f>
         <v/>
       </c>
       <c r="C40" s="14">
-        <f>IF(LEN(detail!X17)&lt;1,"", detail!X17)</f>
-        <v/>
-      </c>
-      <c r="D40" s="31">
-        <f>IF(LEN(detail!R17)&lt;1,"",detail!R17)</f>
-        <v/>
-      </c>
-      <c r="E40" s="30" t="n"/>
+        <f>IF(LEN(detail!X16)&lt;1,"", detail!X16)</f>
+        <v/>
+      </c>
+      <c r="D40" s="37">
+        <f>IF(LEN(detail!R16)&lt;1,"",detail!R16)</f>
+        <v/>
+      </c>
+      <c r="E40" s="36" t="n"/>
       <c r="F40" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF17)&lt;1,"",detail!AF17), 0) &amp; IF(detail!AG17 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G40" s="31">
-        <f>IF(LEN(detail!AC17)&lt;1,"",detail!AC17)</f>
+        <f>DOLLAR(IF(LEN(detail!AF16)&lt;1,"",detail!AF16), 0) &amp; IF(detail!AG16 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G40" s="37">
+        <f>IF(LEN(detail!AC16)&lt;1,"",detail!AC16)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="14">
-        <f>IF(LEN(detail!P18)&lt;1,"",detail!P18)</f>
+        <f>IF(LEN(detail!P17)&lt;1,"",detail!P17)</f>
         <v/>
       </c>
       <c r="C41" s="14">
-        <f>IF(LEN(detail!X18)&lt;1,"", detail!X18)</f>
-        <v/>
-      </c>
-      <c r="D41" s="31">
-        <f>IF(LEN(detail!R18)&lt;1,"",detail!R18)</f>
-        <v/>
-      </c>
-      <c r="E41" s="30" t="n"/>
+        <f>IF(LEN(detail!X17)&lt;1,"", detail!X17)</f>
+        <v/>
+      </c>
+      <c r="D41" s="37">
+        <f>IF(LEN(detail!R17)&lt;1,"",detail!R17)</f>
+        <v/>
+      </c>
+      <c r="E41" s="36" t="n"/>
       <c r="F41" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF18)&lt;1,"",detail!AF18), 0) &amp; IF(detail!AG18 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G41" s="31">
-        <f>IF(LEN(detail!AC18)&lt;1,"",detail!AC18)</f>
+        <f>DOLLAR(IF(LEN(detail!AF17)&lt;1,"",detail!AF17), 0) &amp; IF(detail!AG17 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G41" s="37">
+        <f>IF(LEN(detail!AC17)&lt;1,"",detail!AC17)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="14">
-        <f>IF(LEN(detail!P19)&lt;1,"",detail!P19)</f>
+        <f>IF(LEN(detail!P18)&lt;1,"",detail!P18)</f>
         <v/>
       </c>
       <c r="C42" s="14">
-        <f>IF(LEN(detail!X19)&lt;1,"", detail!X19)</f>
-        <v/>
-      </c>
-      <c r="D42" s="31">
-        <f>IF(LEN(detail!R19)&lt;1,"",detail!R19)</f>
-        <v/>
-      </c>
-      <c r="E42" s="30" t="n"/>
+        <f>IF(LEN(detail!X18)&lt;1,"", detail!X18)</f>
+        <v/>
+      </c>
+      <c r="D42" s="37">
+        <f>IF(LEN(detail!R18)&lt;1,"",detail!R18)</f>
+        <v/>
+      </c>
+      <c r="E42" s="36" t="n"/>
       <c r="F42" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF19)&lt;1,"",detail!AF19), 0) &amp; IF(detail!AG19 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G42" s="31">
-        <f>IF(LEN(detail!AC19)&lt;1,"",detail!AC19)</f>
+        <f>DOLLAR(IF(LEN(detail!AF18)&lt;1,"",detail!AF18), 0) &amp; IF(detail!AG18 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G42" s="37">
+        <f>IF(LEN(detail!AC18)&lt;1,"",detail!AC18)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="14">
-        <f>IF(LEN(detail!P20)&lt;1,"",detail!P20)</f>
+        <f>IF(LEN(detail!P19)&lt;1,"",detail!P19)</f>
         <v/>
       </c>
       <c r="C43" s="14">
-        <f>IF(LEN(detail!X20)&lt;1,"", detail!X20)</f>
-        <v/>
-      </c>
-      <c r="D43" s="31">
-        <f>IF(LEN(detail!R20)&lt;1,"",detail!R20)</f>
-        <v/>
-      </c>
-      <c r="E43" s="30" t="n"/>
+        <f>IF(LEN(detail!X19)&lt;1,"", detail!X19)</f>
+        <v/>
+      </c>
+      <c r="D43" s="37">
+        <f>IF(LEN(detail!R19)&lt;1,"",detail!R19)</f>
+        <v/>
+      </c>
+      <c r="E43" s="36" t="n"/>
       <c r="F43" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF20)&lt;1,"",detail!AF20), 0) &amp; IF(detail!AG20 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G43" s="31">
-        <f>IF(LEN(detail!AC20)&lt;1,"",detail!AC20)</f>
+        <f>DOLLAR(IF(LEN(detail!AF19)&lt;1,"",detail!AF19), 0) &amp; IF(detail!AG19 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G43" s="37">
+        <f>IF(LEN(detail!AC19)&lt;1,"",detail!AC19)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="14">
-        <f>IF(LEN(detail!P21)&lt;1,"",detail!P21)</f>
+        <f>IF(LEN(detail!P20)&lt;1,"",detail!P20)</f>
         <v/>
       </c>
       <c r="C44" s="14">
-        <f>IF(LEN(detail!X21)&lt;1,"", detail!X21)</f>
-        <v/>
-      </c>
-      <c r="D44" s="31">
-        <f>IF(LEN(detail!R21)&lt;1,"",detail!R21)</f>
-        <v/>
-      </c>
-      <c r="E44" s="30" t="n"/>
+        <f>IF(LEN(detail!X20)&lt;1,"", detail!X20)</f>
+        <v/>
+      </c>
+      <c r="D44" s="37">
+        <f>IF(LEN(detail!R20)&lt;1,"",detail!R20)</f>
+        <v/>
+      </c>
+      <c r="E44" s="36" t="n"/>
       <c r="F44" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF21)&lt;1,"",detail!AF21), 0) &amp; IF(detail!AG21 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G44" s="31">
-        <f>IF(LEN(detail!AC21)&lt;1,"",detail!AC21)</f>
+        <f>DOLLAR(IF(LEN(detail!AF20)&lt;1,"",detail!AF20), 0) &amp; IF(detail!AG20 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G44" s="37">
+        <f>IF(LEN(detail!AC20)&lt;1,"",detail!AC20)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="14">
-        <f>IF(LEN(detail!P22)&lt;1,"",detail!P22)</f>
+        <f>IF(LEN(detail!P21)&lt;1,"",detail!P21)</f>
         <v/>
       </c>
       <c r="C45" s="14">
-        <f>IF(LEN(detail!X22)&lt;1,"", detail!X22)</f>
-        <v/>
-      </c>
-      <c r="D45" s="31">
-        <f>IF(LEN(detail!R22)&lt;1,"",detail!R22)</f>
-        <v/>
-      </c>
-      <c r="E45" s="30" t="n"/>
+        <f>IF(LEN(detail!X21)&lt;1,"", detail!X21)</f>
+        <v/>
+      </c>
+      <c r="D45" s="37">
+        <f>IF(LEN(detail!R21)&lt;1,"",detail!R21)</f>
+        <v/>
+      </c>
+      <c r="E45" s="36" t="n"/>
       <c r="F45" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF22)&lt;1,"",detail!AF22), 0) &amp; IF(detail!AG22 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G45" s="31">
-        <f>IF(LEN(detail!AC22)&lt;1,"",detail!AC22)</f>
+        <f>DOLLAR(IF(LEN(detail!AF21)&lt;1,"",detail!AF21), 0) &amp; IF(detail!AG21 = 1, "*", "")</f>
+        <v/>
+      </c>
+      <c r="G45" s="37">
+        <f>IF(LEN(detail!AC21)&lt;1,"",detail!AC21)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="14">
-        <f>IF(LEN(detail!P23)&lt;1,"",detail!P23)</f>
-        <v/>
-      </c>
-      <c r="C46" s="14">
-        <f>IF(LEN(detail!X23)&lt;1,"", detail!X23)</f>
-        <v/>
-      </c>
-      <c r="D46" s="31">
-        <f>IF(LEN(detail!R23)&lt;1,"",detail!R23)</f>
-        <v/>
-      </c>
-      <c r="E46" s="30" t="n"/>
-      <c r="F46" s="9">
-        <f>DOLLAR(IF(LEN(detail!AF23)&lt;1,"",detail!AF23), 0) &amp; IF(detail!AG23 = 1, "*", "")</f>
-        <v/>
-      </c>
-      <c r="G46" s="31">
-        <f>IF(LEN(detail!AC23)&lt;1,"",detail!AC23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="1" t="inlineStr">
+      <c r="B46" s="39" t="inlineStr">
         <is>
           <t>* An asterisk denotes that the opp includes a rebate</t>
         </is>
@@ -1929,9 +1955,8 @@
   <mergeCells count="37">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="E9:G9"/>
-    <mergeCell ref="D46:E46"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="D36:E36"/>
@@ -1940,12 +1965,13 @@
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E10:F10"/>
+    <mergeCell ref="D27:E27"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="D27:E27"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B24:G24"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="E11:F11"/>
@@ -1954,20 +1980,20 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D25:E25"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="E16:F16"/>
     <mergeCell ref="D42:E42"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="D38:E38"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D35:E35"/>
   </mergeCells>
-  <conditionalFormatting sqref="B25:D46 F25:G46">
+  <conditionalFormatting sqref="B26:D45 F26:G45">
     <cfRule type="containsErrors" priority="1" dxfId="0">
-      <formula>ISERROR(B25)</formula>
+      <formula>ISERROR(B26)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2035,7 +2061,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2054,7 +2080,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>123000</v>
+        <v>0</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2070,7 +2096,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2089,7 +2115,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2105,7 +2131,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2124,7 +2150,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2140,7 +2166,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2159,7 +2185,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>63000</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2175,7 +2201,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2194,7 +2220,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>9450</v>
+        <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2210,7 +2236,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2245,7 +2271,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2280,7 +2306,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2299,7 +2325,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2315,7 +2341,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2350,7 +2376,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2385,7 +2411,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2404,7 +2430,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>18950</v>
+        <v>250</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2420,7 +2446,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2439,7 +2465,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>16666.67</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -2455,7 +2481,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2474,7 +2500,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>18950</v>
+        <v>16666.67</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -2490,7 +2516,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2509,7 +2535,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -2525,7 +2551,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2544,7 +2570,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -2560,7 +2586,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2579,7 +2605,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>123000</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2595,7 +2621,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2630,7 +2656,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2649,7 +2675,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>18950</v>
+        <v>16667</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -2668,7 +2694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.5703125" customWidth="1" min="1" max="1"/>
@@ -2683,7 +2709,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Jennifer Malberg</t>
+          <t>David Solomon</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2721,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>jmalberg@cvrx.com</t>
+          <t>dsolomon@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2733,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mbrown@cvrx.com</t>
+          <t>dhoman@cvrx.com</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2745,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NORTH CALIFORNIA (MALBERG)</t>
+          <t>ARKANSAS (SOLOMON)</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2780,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>170362.5</v>
+        <v>148500</v>
       </c>
     </row>
     <row r="8">
@@ -2764,7 +2790,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>245322</v>
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Recoverable Draw:</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>51083.34</v>
       </c>
     </row>
     <row r="21" ht="15.95" customHeight="1"/>
@@ -2782,7 +2818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU4"/>
+  <dimension ref="A1:AU1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3022,530 +3058,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Jennifer Malberg</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PACIFIC</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>RE_07</t>
-        </is>
-      </c>
-      <c r="I2" s="52" t="n">
-        <v>46048</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026_01</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026_01</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>University of California Health (AKA UC Health-CA)</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Ucsf Medical Center</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>0014u00001pyZlqAAE</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>CVR314 028890</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>006UY00000U3JknYAF</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Heart Failure - Reduced Ejection Fraction</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>De novo</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Revenue Recognized</t>
-        </is>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>170362.5</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>245322</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>4725</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Jennifer Malberg</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PACIFIC</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>RE_07</t>
-        </is>
-      </c>
-      <c r="I3" s="52" t="n">
-        <v>46048</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026_01</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026_01</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>University of California Health (AKA UC Health-CA)</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Ucsf Medical Center</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>0014u00001pyZlqAAE</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>CVR314 029551</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>006UY00000VfcIoYAJ</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Heart Failure - Reduced Ejection Fraction</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>De novo</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Revenue Recognized</t>
-        </is>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>170362.5</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>245322</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>63000</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>31500</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>4725</v>
-      </c>
-      <c r="AU3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Jennifer Malberg</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TERR_37</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PACIFIC</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>RE_07</t>
-        </is>
-      </c>
-      <c r="I4" s="52" t="n">
-        <v>46053</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2026_01</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026_02</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026_Q1</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Kaweah Health (FKA Kaweah Delta Health Care District)</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Kaweah Delta Medical Center</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>0014u00001s9EpwAAE</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>CRX305 029860</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>006UY00000WRIhZYAX</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>jmalberg@cvrx.com</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Heart Failure - Reduced Ejection Fraction</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>De novo</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Revenue Recognized</t>
-        </is>
-      </c>
-      <c r="Z4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>60000</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>60000</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>30000</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>170362.5</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>245322</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>123000</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>brummonds@cvrx.com</t>
-        </is>
-      </c>
-      <c r="AO4" t="n">
-        <v>60000</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>9000</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>